<commit_message>
Make the Instagram plan faceless with step-by-step production for every post
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vRai2Js1dvdXXwRHYcreT
</commit_message>
<xml_diff>
--- a/marginwise/instagram-content-calendar.xlsx
+++ b/marginwise/instagram-content-calendar.xlsx
@@ -11,12 +11,13 @@
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Calendar" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Stories" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Filming batches" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Weekly review" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Setup before 14 Oct" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="How to make (no face)" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Recording batches" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Weekly review" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Setup before 14 Oct" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$Y$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$Z$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="258">
   <si>
     <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 15 Nov 2026</t>
   </si>
@@ -39,13 +40,16 @@
     <t xml:space="preserve">Tabs</t>
   </si>
   <si>
-    <t xml:space="preserve">Calendar: every post with hook, outline, caption, CTA keyword and lead magnet. Fill the yellow columns after posting.</t>
+    <t xml:space="preserve">Calendar: every post with hook, outline, step-by-step production (faceless), caption, CTA keyword and lead magnet. Fill the yellow columns after posting.</t>
   </si>
   <si>
     <t xml:space="preserve">Stories: the weekly Stories rhythm.</t>
   </si>
   <si>
-    <t xml:space="preserve">Filming batches: what to film in each session so you are never filming the night before.</t>
+    <t xml:space="preserve">How to make (no face): the kit and the step-by-step method used for every post. No camera needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recording batches: what to record in each session so you are never recording the night before.</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly review: totals per week, calculated from the Calendar tab.</t>
@@ -108,6 +112,9 @@
     <t xml:space="preserve">Outline</t>
   </si>
   <si>
+    <t xml:space="preserve">Step by step (no face)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Caption</t>
   </si>
   <si>
@@ -123,7 +130,7 @@
     <t xml:space="preserve">Pin?</t>
   </si>
   <si>
-    <t xml:space="preserve">Filming batch</t>
+    <t xml:space="preserve">Recording batch</t>
   </si>
   <si>
     <t xml:space="preserve">Status</t>
@@ -171,15 +178,24 @@
     <t xml:space="preserve">Both</t>
   </si>
   <si>
-    <t xml:space="preserve">Every agency sells you ROAS. I sell you margin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Who I am: 10 years building D2C, omnichannel and loyalty products. 2) The four services in one line each. 3) Who it is not for: pre-launch ideas, single theme tweaks, guaranteed-results deals. 4) How the free 30-min call works and what you leave with.</t>
+    <t xml:space="preserve">Every agency sells you ROAS. We sell you margin. This is what that looks like.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen walkthrough of a Marginwise audit on a demo store (your own Shopify dev store or a public store, no client data): 1) funnel numbers, 2) three leaks ranked by revenue impact, 3) the one fix to ship this week, 4) the written summary the founder gets. Close on the four services and who it is not for.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record (desktop, QuickTime or OBS, 1080p) a walkthrough of an audit on a demo store: GA4 funnel, three leaks marked in a doc, the one-page written summary. Use a Shopify dev store or public pages only.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Open with: 'This is what we look at before we touch your ads.'
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Zoom (keyframes) on each leak as you name it; red box highlights. Pin this post after publishing.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Most agencies report ROAS. We report what you keep.
-Marginwise runs CRO, performance marketing, UX and app development for D2C and Shopify brands in India, the US and the UK. Every engagement starts with a free 30-minute call: you leave with your top three leaks and a written summary.
-Comment AUDIT and I will send you a 2-minute teardown of your store.
+This is what a Marginwise audit looks like: your funnel, your three biggest leaks ranked by revenue impact, one fix to ship this week, and a written summary.
+CRO, performance marketing, UX and app development for D2C and Shopify brands in India, the US and the UK.
+Comment AUDIT and we will send you a 2-minute teardown of your store.
 #d2c #shopify #ecommercegrowth</t>
   </si>
   <si>
@@ -219,8 +235,16 @@
     <t xml:space="preserve">Show 3x ROAS on screen. Remove over-attribution, returns, COGS, shipping, payment fees one by one. Land on contribution after ads. End: track contribution margin per order, not ROAS.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator (ROAS to Profit tab) at 150% zoom, typing in a 3x ROAS store and watching contribution turn negative.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Say each cost as it is subtracted; end on the break-even ROAS cell.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the cell being changed each time; end frame on the verdict cell.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROAS is not profit. Here is what a 3x ROAS can actually leave you with once over-attribution, returns, product cost, shipping and fees come out.
-Comment PROFIT and I will send you the calculator to run it on your own numbers.
+Comment PROFIT and we will send you the calculator to run it on your own numbers.
 #shopify #metaads #dtc</t>
   </si>
   <si>
@@ -240,6 +264,14 @@
   </si>
   <si>
     <t xml:space="preserve">S1 hook. S2 70.22% of carts abandoned (Baymard). S3 35% conversion gain from better checkout design (Baymard). S4 8.4% more conversions from 0.1s faster mobile (Deloitte/Google). S5 26% RTO on COD vs under 2% prepaid (Shipway FY25). S6 what to fix first. S7 CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. Big number top half, one-line meaning and 'what to fix' bottom half.
+3. Put a source line (small, bottom) on every slide with a statistic.
+4. Last slide: CTA with the comment keyword in large text.
+5. Export as PNG, upload in order, add alt text to slide 1.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Four published numbers that explain where most D2C stores lose revenue, and what to fix first for each. Sources on every slide.
@@ -268,8 +300,16 @@
     <t xml:space="preserve">Shipway FY25: 26% RTO on COD vs under 2% prepaid. What one RTO costs: forward and return shipping, packaging, wasted ad spend. Three fixes: prepaid incentive, WhatsApp confirmation for risky COD, switch off COD only in high-RTO pin codes.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the RTO finder with sample orders loaded: the By State tab sorting by cost, one state flagged 'Restrict COD or verify'.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Use the Shipway 26% vs under 2% figure in the first line.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text callout for each of the three fixes as you say it.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Switching off COD everywhere is the wrong fix. Find the pin codes where it loses money and act only there.
-Comment RTO and I will send you the sheet that ranks your states and pin codes by RTO cost.
+Comment RTO and we will send you the sheet that ranks your states and pin codes by RTO cost.
 #d2cindia #rto #shopifyindia</t>
   </si>
   <si>
@@ -289,6 +329,14 @@
   </si>
   <si>
     <t xml:space="preserve">Screen-record a well-known US/UK brand's mobile product page. Two strengths, one leak (hidden shipping cost, review placement, or slow image). What that leak costs in margin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record (iOS Control Centre &gt; Screen Recording, or Android quick settings) the brand's mobile product page: scroll slowly, add to cart, open cart. 40 seconds, no notifications (Do Not Disturb on).
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Two things it does well, then the one leak and what it costs.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red circle on the leak; slow-zoom into it. Blur any personal data.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">A product page teardown with a margin lens: what converts, what leaks, and what the leak costs.
@@ -305,8 +353,16 @@
     <t xml:space="preserve">Break down a ₹1,000 order: GST, COGS, ad cost per order, shipping, RTO, gateway fees, discounts. Land on contribution margin per order. Investors now ask for this, not GMV.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the MARGIN calculator, Margin per Order tab, stepping through each cost line of a ₹1,000 order.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. One sentence per cost line; end on contribution per order.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Running total as on-screen text in the top corner.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Contribution margin per order, explained with a real ₹1,000 example.
-Comment MARGIN and I will send you the calculator, including a what-if for pushing more buyers to prepaid.
+Comment MARGIN and we will send you the calculator, including a what-if for pushing more buyers to prepaid.
 #d2cindia #unitEconomics #founders</t>
   </si>
   <si>
@@ -323,6 +379,14 @@
   </si>
   <si>
     <t xml:space="preserve">One cost per slide: GST, product cost, ad cost, shipping and packaging, RTO, COD fees, gateway fees. Final slide: contribution per order and the one lever that moves it most.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. One cost per slide with the running total shown on every slide.
+3. Put a source line (small, bottom) on every slide with a statistic.
+4. Last slide: CTA with the comment keyword in large text.
+5. Export as PNG, upload in order, add alt text to slide 1.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Line by line, what is left of a ₹1,000 order once every cost is counted. Numbers are an example store; run your own with the calculator.
@@ -339,6 +403,14 @@
     <t xml:space="preserve">Five public checkouts (mix of US/UK and Indian). One thing each does well: trust badges placement, delivery date, COD/prepaid nudge, express pay, order summary clarity.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Phone screen-record five public checkouts (stop before payment). 6-8 seconds each.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. One line per checkout: what it does well.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Numbered label 1-5 on screen; 'Save this' text on the final frame.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Five checkouts worth studying before your next redesign, and the one thing each gets right.
 Save this. Comment AUDIT if you want yours reviewed.
 #checkout #shopify #cro</t>
@@ -353,6 +425,14 @@
     <t xml:space="preserve">Baymard: 70.22% average cart abandonment across 50 studies. Three fixable reasons: surprise costs, forced account creation, too many steps. Show one fix for each on a Shopify checkout.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Phone screen-record a checkout showing a surprise shipping cost, a forced account screen and a long form (public stores).
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Lead with Baymard's 70.22%; one fix per problem.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Split screen: problem on top, fix described as text below.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cart abandonment averages 70% (Baymard Institute). Three fixes that do not need a redesign.
 Save this for your next checkout review.
 #checkout #shopifytips #ecommerce</t>
@@ -373,6 +453,14 @@
     <t xml:space="preserve">Screen-record an Indian D2C brand's mobile product page. Two strengths, one leak (COD/prepaid messaging, delivery date clarity, size guidance). The fix.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Phone screen-record the Indian brand's mobile product page: price, delivery date, COD/prepaid messaging, size guide.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Two strengths, one leak, the fix.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red circle on the leak; ₹ figures as on-screen text.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">A mobile product page teardown of an Indian D2C brand, and one fix that lifts conversion without a redesign.
 Comment AUDIT for a teardown of your store.
 #d2cindia #cro #shopifyindia</t>
@@ -387,6 +475,14 @@
     <t xml:space="preserve">S1 hook. S2 overlap hours (your morning, our evening). S3 weekly written update, with redacted example. S4 one senior contact. S5 billing in USD/GBP, NDA, 30-day notice. S6 CTA.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. Slide 3 shows a redacted sample weekly update; build it from a blank template, not client data.
+3. Put a source line (small, bottom) on every slide with a statistic.
+4. Last slide: CTA with the comment keyword in large text.
+5. Export as PNG, upload in order, add alt text to slide 1.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The three things founders worry about with an offshore team, and exactly how we handle each one.
 See how we work at the link in bio.
 #ecommerceagency #shopifyexperts #dtc</t>
@@ -404,6 +500,14 @@
     <t xml:space="preserve">Communication, time zones, quality. How each should be handled by any agency: overlap hours, weekly written update, one senior point of contact. 'Ask any agency for these three.'</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF scrolling to the 'If the agency is in another country' section, plus a world clock showing IST vs ET overlap.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Name the three worries, then the three answers.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text list builds one line at a time.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">What to ask any offshore agency before you sign, ourselves included.
 Comment CHECKLIST for the full agency hiring checklist.
 #ecommerceagency #shopify #dtcbrands</t>
@@ -424,6 +528,14 @@
     <t xml:space="preserve">Rate three order confirmation emails (public or redacted) with a score and one reason each. End on what a 9/10 email contains.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screenshot three order confirmation emails (your own inbox; blur names, order numbers, addresses).
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Score each out of 10 with one reason; end on what a 9/10 has.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Big score number appears on each email; slow scroll down each one.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Your order confirmation email is the most-opened email you send. Most brands waste it on a receipt.
 Comment FLOWS for the post-purchase checklist and a 10-point scorecard.
 #klaviyo #emailmarketing #dtc</t>
@@ -441,8 +553,16 @@
     <t xml:space="preserve">Deloitte/Google study of 37 brands. Run a public store through PageSpeed. Show the three usual culprits: app scripts, oversized images, third-party widgets. Fix speed before buying more traffic.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record pagespeed.web.dev running on a public Shopify store, then the opportunities list.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Lead with Deloitte/Google 0.1s = 8.4%; name the three culprits.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the three culprits in the report as you name them.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fix speed before you buy more traffic. The three culprits on most Shopify stores.
-Comment SPEED and I will check your store.
+Comment SPEED and we will check your store.
 #shopifyspeed #cro #ecommerce</t>
   </si>
   <si>
@@ -456,6 +576,14 @@
   </si>
   <si>
     <t xml:space="preserve">One fix per slide: shipping cost shown early, guest checkout, express pay, delivery date, stock and promo messaging, mobile speed, post-purchase upsell that keeps margin. Final slide CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. One fix per slide with a small mock of the checkout element it refers to.
+3. Put a source line (small, bottom) on every slide with a statistic.
+4. Last slide: CTA with the comment keyword in large text.
+5. Export as PNG, upload in order, add alt text to slide 1.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Seven checkout fixes you can still ship before Black Friday, none of which need a redesign.
@@ -469,6 +597,14 @@
     <t xml:space="preserve">Who works on my account? Whose name is the ad account in? Show a redacted report with CPA. Notice period? Which one metric in month one?</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF, top table (five questions, good answer, red flag).
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Read each question and its red flag.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight each row as you read it.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Most founders pick an agency from the pitch deck. Ask these five questions instead, including to us.
 Comment CHECKLIST for the full list.
 #d2c #marketingagency #founders</t>
@@ -480,6 +616,14 @@
     <t xml:space="preserve">Since the $800 de minimis exemption ended, landed costs rose. Landed cost before and after (illustrative). Three levers besides price: AOV bundles, free-shipping threshold, push higher-margin products.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator with COGS raised to show a tariff hit, then bundle/AOV changes recovering margin.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Before vs after landed cost; three levers.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Before/after numbers side by side as text.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rising import costs hit contribution margin first. Three ways to protect it without a price rise.
 Comment PROFIT for the margin calculator.
 #dtc #tariffs #shopify</t>
@@ -497,6 +641,14 @@
     <t xml:space="preserve">Meta Ireland billing means 18% GST under reverse charge, paid in cash before credit. Show the cash timing. Add 18% to the ad budget in your cash-flow plan. Confirm with your CA.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Record: Screen-record the MARGIN calculator, GST on Ads tab, typing ₹1,00,000.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Explain reverse charge in one sentence; say 'confirm with your CA'.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Show '₹1,18,000 leaves your account' as the final frame.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The GST line that catches founders short on cash. Not tax advice; confirm with your CA.
 Comment MARGIN for the calculator, which includes a GST-on-ads tab.
 #d2cindia #metaads #gst</t>
@@ -508,15 +660,31 @@
     <t xml:space="preserve">S1 hook. S2 why sale buyers churn. S3 the delivered + how-to-use email. S4 review request timing. S5 replenishment timed to your data. S6 win-back without a discount first. S7 CTA.</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. Each email slide shows when to send it and one line of example copy.
+3. Put a source line (small, bottom) on every slide with a statistic.
+4. Last slide: CTA with the comment keyword in large text.
+5. Export as PNG, upload in order, add alt text to slide 1.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sale buyers are the easiest to lose. Five emails that bring them back without giving away margin.
 Comment FLOWS for the full checklist.
 #retention #emailmarketing #d2c</t>
   </si>
   <si>
-    <t xml:space="preserve">I audited [N] D2C stores this month. The same 3 leaks showed up in [X] of them.</t>
+    <t xml:space="preserve">We audited [N] D2C stores this month. The same 3 leaks showed up in [X] of them.</t>
   </si>
   <si>
     <t xml:space="preserve">Only post if the audits are real; use the actual count. Three most common leaks, anonymised. If fewer than 5 audits are done, swap for a second Indian teardown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a tally sheet of the audits you actually ran (store names hidden) and anonymised screenshots of the three leaks.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Use the real count. If under 5 audits, swap for a second Indian teardown and follow that recipe.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Counter animation for each leak's tally.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">What we keep finding when we audit D2C stores, with no names attached.
@@ -584,12 +752,72 @@
     <t xml:space="preserve">Answer</t>
   </si>
   <si>
-    <t xml:space="preserve">Answer one question from DMs or the question box on camera (30-45s).</t>
+    <t xml:space="preserve">Answer one question from DMs as 2-3 text frames over a screen recording or screenshot of the relevant page.</t>
   </si>
   <si>
     <t xml:space="preserve">Turns DMs into content and shows you reply.</t>
   </si>
   <si>
+    <t xml:space="preserve">Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop with QuickTime (Mac) or OBS (Windows) for desktop recording; phone screen recorder; CapCut (free); Canva (free); wired earphones with mic or any USB mic. No camera needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before recording</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do Not Disturb on, browser in a clean profile (no bookmarks, no logged-in personal accounts), zoom browser to 125-150% so text is readable on a phone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recording</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Move the cursor slowly and pause 1 second on anything you will talk about. Record 20% more than you need.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voiceover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your own voice, phone held 15 cm away, in a room with soft furnishings. Read from the script, then do one natural take without reading; use whichever sounds less scripted. Instagram rewards real human content; skip AI voices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you do not want to use your voice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text-only version: put each script line as a caption block (3-4 words per screen), add quiet background music from CapCut's commercial library. Expect lower watch time; test it as a Trial Reel first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CapCut: 9:16, Auto captions, hook text in the first 2 seconds, cut every pause over half a second, zoom and red-box highlights on whatever you name. Length 30-60 seconds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blur names, emails, order numbers and any client data. Teardowns use public pages only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canva 1080x1350, one template for all, max 25 words per slide, source line on stat slides, CTA slide last.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After posting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reply to every comment in the first hour; check the auto-DM fired; log numbers in the Calendar tab after 7 days.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Batch</t>
   </si>
   <si>
@@ -608,7 +836,7 @@
     <t xml:space="preserve">Founder intro; ROAS 3x; COD RTO 26%; US/UK product page teardown; ₹1,000 order margin; 5 checkout pages</t>
   </si>
   <si>
-    <t xml:space="preserve">Pick the US/UK brand and 5 checkouts (public pages). Screen recordings done before filming. Same shirt across takes to batch-edit.</t>
+    <t xml:space="preserve">Pick the US/UK brand and 5 checkouts (public pages). Record all screen captures first, then write and record every voiceover in one sitting.</t>
   </si>
   <si>
     <t xml:space="preserve">3 hours</t>
@@ -1288,7 +1516,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1309,7 +1537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1335,16 +1563,16 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1365,8 +1593,13 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1385,7 +1618,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1398,99 +1631,103 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="21" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
@@ -1498,62 +1735,65 @@
         <v>46309</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S2" s="9"/>
-      <c r="T2" s="10"/>
+        <v>57</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T2" s="9"/>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
       <c r="W2" s="10"/>
       <c r="X2" s="10"/>
       <c r="Y2" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
@@ -1561,62 +1801,65 @@
         <v>46311</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P3" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G3" s="6" t="s">
+      <c r="Q3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="R3" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" s="9"/>
-      <c r="T3" s="10"/>
+      <c r="T3" s="9"/>
       <c r="U3" s="10"/>
       <c r="V3" s="10"/>
       <c r="W3" s="10"/>
       <c r="X3" s="10"/>
       <c r="Y3" s="10"/>
-    </row>
-    <row r="4" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
@@ -1624,62 +1867,65 @@
         <v>46312</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="S4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q4" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="R4" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S4" s="9"/>
-      <c r="T4" s="10"/>
+      <c r="T4" s="9"/>
       <c r="U4" s="10"/>
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
       <c r="X4" s="10"/>
       <c r="Y4" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
@@ -1687,62 +1933,65 @@
         <v>46313</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S5" s="9"/>
-      <c r="T5" s="10"/>
+        <v>57</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T5" s="9"/>
       <c r="U5" s="10"/>
       <c r="V5" s="10"/>
       <c r="W5" s="10"/>
       <c r="X5" s="10"/>
       <c r="Y5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
         <v>2</v>
       </c>
@@ -1750,62 +1999,65 @@
         <v>46315</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S6" s="9"/>
-      <c r="T6" s="10"/>
+        <v>57</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T6" s="9"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
       <c r="W6" s="10"/>
       <c r="X6" s="10"/>
       <c r="Y6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
         <v>2</v>
       </c>
@@ -1813,62 +2065,65 @@
         <v>46317</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H7" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="P7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S7" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q7" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="R7" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S7" s="9"/>
-      <c r="T7" s="10"/>
+      <c r="T7" s="9"/>
       <c r="U7" s="10"/>
       <c r="V7" s="10"/>
       <c r="W7" s="10"/>
       <c r="X7" s="10"/>
       <c r="Y7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
         <v>2</v>
       </c>
@@ -1876,62 +2131,65 @@
         <v>46319</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="H8" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="S8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P8" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q8" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="R8" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S8" s="9"/>
-      <c r="T8" s="10"/>
+      <c r="T8" s="9"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
       <c r="W8" s="10"/>
       <c r="X8" s="10"/>
       <c r="Y8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
         <v>2</v>
       </c>
@@ -1939,62 +2197,65 @@
         <v>46320</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q9" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="R9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="O9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="P9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q9" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="R9" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S9" s="9"/>
-      <c r="T9" s="10"/>
+      <c r="S9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T9" s="9"/>
       <c r="U9" s="10"/>
       <c r="V9" s="10"/>
       <c r="W9" s="10"/>
       <c r="X9" s="10"/>
       <c r="Y9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
@@ -2002,62 +2263,65 @@
         <v>46322</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>53</v>
+        <v>115</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S10" s="9"/>
-      <c r="T10" s="10"/>
+        <v>116</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T10" s="9"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10"/>
       <c r="W10" s="10"/>
       <c r="X10" s="10"/>
       <c r="Y10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
         <v>3</v>
       </c>
@@ -2065,62 +2329,65 @@
         <v>46324</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S11" s="9"/>
-      <c r="T11" s="10"/>
+        <v>116</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T11" s="9"/>
       <c r="U11" s="10"/>
       <c r="V11" s="10"/>
       <c r="W11" s="10"/>
       <c r="X11" s="10"/>
       <c r="Y11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>3</v>
       </c>
@@ -2128,62 +2395,65 @@
         <v>46326</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S12" s="9"/>
-      <c r="T12" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T12" s="9"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
       <c r="W12" s="10"/>
       <c r="X12" s="10"/>
       <c r="Y12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
         <v>3</v>
       </c>
@@ -2191,62 +2461,65 @@
         <v>46327</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="K13" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="R13" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="L13" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="P13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q13" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="R13" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S13" s="9"/>
-      <c r="T13" s="10"/>
+      <c r="S13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T13" s="9"/>
       <c r="U13" s="10"/>
       <c r="V13" s="10"/>
       <c r="W13" s="10"/>
       <c r="X13" s="10"/>
       <c r="Y13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="n">
         <v>4</v>
       </c>
@@ -2254,62 +2527,65 @@
         <v>46329</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>53</v>
+        <v>140</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="Q14" s="11" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="R14" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S14" s="9"/>
-      <c r="T14" s="10"/>
+        <v>116</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T14" s="9"/>
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
       <c r="W14" s="10"/>
       <c r="X14" s="10"/>
       <c r="Y14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
         <v>4</v>
       </c>
@@ -2317,62 +2593,65 @@
         <v>46331</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>52</v>
+        <v>146</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="R15" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S15" s="9"/>
-      <c r="T15" s="10"/>
+        <v>116</v>
+      </c>
+      <c r="S15" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T15" s="9"/>
       <c r="U15" s="10"/>
       <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
         <v>4</v>
       </c>
@@ -2380,62 +2659,65 @@
         <v>46333</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P16" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q16" s="11" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="R16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S16" s="9"/>
-      <c r="T16" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="S16" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T16" s="9"/>
       <c r="U16" s="10"/>
       <c r="V16" s="10"/>
       <c r="W16" s="10"/>
       <c r="X16" s="10"/>
       <c r="Y16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
         <v>4</v>
       </c>
@@ -2443,62 +2725,65 @@
         <v>46334</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q17" s="11" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
       <c r="R17" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="S17" s="9"/>
-      <c r="T17" s="10"/>
+        <v>116</v>
+      </c>
+      <c r="S17" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T17" s="9"/>
       <c r="U17" s="10"/>
       <c r="V17" s="10"/>
       <c r="W17" s="10"/>
       <c r="X17" s="10"/>
       <c r="Y17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
         <v>5</v>
       </c>
@@ -2506,62 +2791,65 @@
         <v>46336</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H18" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="S18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="O18" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q18" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="R18" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S18" s="9"/>
-      <c r="T18" s="10"/>
+      <c r="T18" s="9"/>
       <c r="U18" s="10"/>
       <c r="V18" s="10"/>
       <c r="W18" s="10"/>
       <c r="X18" s="10"/>
       <c r="Y18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="n">
         <v>5</v>
       </c>
@@ -2569,62 +2857,65 @@
         <v>46338</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="H19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="S19" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="O19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="P19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q19" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="R19" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S19" s="9"/>
-      <c r="T19" s="10"/>
+      <c r="T19" s="9"/>
       <c r="U19" s="10"/>
       <c r="V19" s="10"/>
       <c r="W19" s="10"/>
       <c r="X19" s="10"/>
       <c r="Y19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z19" s="10"/>
+    </row>
+    <row r="20" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
         <v>5</v>
       </c>
@@ -2632,62 +2923,65 @@
         <v>46340</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>124</v>
+        <v>168</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>52</v>
+        <v>140</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S20" s="9"/>
-      <c r="T20" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T20" s="9"/>
       <c r="U20" s="10"/>
       <c r="V20" s="10"/>
       <c r="W20" s="10"/>
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Z20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="n">
         <v>5</v>
       </c>
@@ -2695,65 +2989,68 @@
         <v>46341</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>50</v>
+        <v>172</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P21" s="6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>140</v>
+        <v>55</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="S21" s="9"/>
-      <c r="T21" s="10"/>
+        <v>159</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="T21" s="9"/>
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
       <c r="W21" s="10"/>
       <c r="X21" s="10"/>
       <c r="Y21" s="10"/>
+      <c r="Z21" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y21"/>
+  <autoFilter ref="A1:Z21"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="R2:R21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="S2:S21" type="list">
       <formula1>"Planned,Filmed,Edited,Scheduled,Posted,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2786,87 +3083,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -2885,6 +3182,109 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2897,87 +3297,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>173</v>
+        <v>215</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>174</v>
+        <v>216</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>175</v>
+        <v>217</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>176</v>
+        <v>218</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>177</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46308</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>178</v>
+        <v>220</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>179</v>
+        <v>221</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>180</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46319</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>181</v>
+        <v>223</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>182</v>
+        <v>224</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>180</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46333</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>183</v>
+        <v>225</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>185</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>46310</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>186</v>
+        <v>228</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>187</v>
+        <v>229</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>188</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2991,7 +3391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3012,40 +3412,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>189</v>
+        <v>231</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>190</v>
+        <v>232</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>191</v>
+        <v>233</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>192</v>
+        <v>234</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>193</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3060,31 +3460,31 @@
         <v>4</v>
       </c>
       <c r="D2" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A2,Calendar!$R$2:$R$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A2,Calendar!$S$2:$S$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$T$2:$T$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$U$2:$U$21)</f>
         <v>0</v>
       </c>
       <c r="F2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="G2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="H2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="I2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="J2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="K2" s="17" t="n">
@@ -3105,31 +3505,31 @@
         <v>4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A3,Calendar!$R$2:$R$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A3,Calendar!$S$2:$S$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$T$2:$T$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$U$2:$U$21)</f>
         <v>0</v>
       </c>
       <c r="F3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="G3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="H3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="I3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="J3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="K3" s="17" t="n">
@@ -3150,31 +3550,31 @@
         <v>4</v>
       </c>
       <c r="D4" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A4,Calendar!$R$2:$R$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A4,Calendar!$S$2:$S$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$T$2:$T$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$U$2:$U$21)</f>
         <v>0</v>
       </c>
       <c r="F4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="G4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="H4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="I4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="J4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="K4" s="17" t="n">
@@ -3195,31 +3595,31 @@
         <v>4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A5,Calendar!$R$2:$R$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A5,Calendar!$S$2:$S$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$T$2:$T$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$U$2:$U$21)</f>
         <v>0</v>
       </c>
       <c r="F5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="G5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="H5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="I5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="J5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="K5" s="17" t="n">
@@ -3240,31 +3640,31 @@
         <v>4</v>
       </c>
       <c r="D6" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A6,Calendar!$R$2:$R$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A6,Calendar!$S$2:$S$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$T$2:$T$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$U$2:$U$21)</f>
         <v>0</v>
       </c>
       <c r="F6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="G6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="H6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="I6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="J6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="K6" s="17" t="n">
@@ -3275,7 +3675,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>194</v>
+        <v>236</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUM(C2:C6)</f>
@@ -3316,7 +3716,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>195</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -3330,7 +3730,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3345,94 +3745,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>196</v>
+        <v>238</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>197</v>
+        <v>239</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22"/>
       <c r="B2" s="6" t="s">
-        <v>198</v>
+        <v>240</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>199</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
-        <v>200</v>
+        <v>242</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>201</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22"/>
       <c r="B4" s="6" t="s">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>203</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22"/>
       <c r="B5" s="6" t="s">
-        <v>204</v>
+        <v>246</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>205</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="6" t="s">
-        <v>206</v>
+        <v>248</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>207</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
-        <v>208</v>
+        <v>250</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>209</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
-        <v>210</v>
+        <v>252</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>211</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
-        <v>212</v>
+        <v>254</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>213</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="6" t="s">
-        <v>214</v>
+        <v>256</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>215</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add checklist PDFs for every Instagram keyword and a BFCM keyword
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vRai2Js1dvdXXwRHYcreT
</commit_message>
<xml_diff>
--- a/marginwise/instagram-content-calendar.xlsx
+++ b/marginwise/instagram-content-calendar.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="260">
   <si>
     <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 15 Nov 2026</t>
   </si>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">AUDIT</t>
   </si>
   <si>
-    <t xml:space="preserve">Free 2-min teardown (manual)</t>
+    <t xml:space="preserve">marginwise-store-leak-audit.pdf + free 2-min teardown</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -251,7 +251,7 @@
     <t xml:space="preserve">PROFIT</t>
   </si>
   <si>
-    <t xml:space="preserve">marginwise-profit-calculator-usd.xlsx</t>
+    <t xml:space="preserve">marginwise-profit-calculator-usd.xlsx + marginwise-roas-to-profit-checklist.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Sat</t>
@@ -316,7 +316,7 @@
     <t xml:space="preserve">RTO</t>
   </si>
   <si>
-    <t xml:space="preserve">marginwise-rto-finder.xlsx</t>
+    <t xml:space="preserve">marginwise-rto-finder.xlsx + marginwise-cod-rto-playbook.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Tue</t>
@@ -369,7 +369,7 @@
     <t xml:space="preserve">MARGIN</t>
   </si>
   <si>
-    <t xml:space="preserve">marginwise-margin-calculator-inr.xlsx</t>
+    <t xml:space="preserve">marginwise-margin-calculator-inr.xlsx + marginwise-contribution-margin-checklist.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Carousel (8 slides)</t>
@@ -569,7 +569,7 @@
     <t xml:space="preserve">SPEED</t>
   </si>
   <si>
-    <t xml:space="preserve">Speed check (manual)</t>
+    <t xml:space="preserve">marginwise-shopify-speed-checklist.pdf + speed check</t>
   </si>
   <si>
     <t xml:space="preserve">Black Friday checkout checklist: 7 fixes before 27 November</t>
@@ -587,8 +587,14 @@
   </si>
   <si>
     <t xml:space="preserve">Seven checkout fixes you can still ship before Black Friday, none of which need a redesign.
-Save this. Comment AUDIT if you want us to check yours before the sale.
+Save this. Comment BFCM for the full checklist with a sale timeline.
 #blackfriday #bfcm #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFCM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marginwise-black-friday-checklist.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Five questions to ask before you hire a D2C agency.</t>
@@ -911,13 +917,13 @@
     <t xml:space="preserve">A hacked brand account is hard to recover</t>
   </si>
   <si>
-    <t xml:space="preserve">Five lead magnets uploaded (Drive or website) with share links</t>
+    <t xml:space="preserve">All lead magnets (3 sheets, 8 PDFs) uploaded to Drive or the website with share links</t>
   </si>
   <si>
     <t xml:space="preserve">Every CTA keyword depends on these</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto-DM tool connected and the 7 keywords tested from a second account</t>
+    <t xml:space="preserve">Auto-DM tool connected and the 8 keywords tested from a second account</t>
   </si>
   <si>
     <t xml:space="preserve">Broken DMs waste the first reels</t>
@@ -2692,10 +2698,10 @@
         <v>150</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>53</v>
+        <v>151</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>54</v>
+        <v>152</v>
       </c>
       <c r="P16" s="11" t="s">
         <v>55</v>
@@ -2746,16 +2752,16 @@
         <v>79</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="N17" s="11" t="s">
         <v>132</v>
@@ -2812,16 +2818,16 @@
         <v>62</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="N18" s="6" t="s">
         <v>67</v>
@@ -2836,7 +2842,7 @@
         <v>55</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="S18" s="6" t="s">
         <v>58</v>
@@ -2869,7 +2875,7 @@
         <v>104</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>61</v>
@@ -2878,16 +2884,16 @@
         <v>79</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="N19" s="6" t="s">
         <v>97</v>
@@ -2902,7 +2908,7 @@
         <v>55</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="S19" s="6" t="s">
         <v>58</v>
@@ -2944,16 +2950,16 @@
         <v>48</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="N20" s="6" t="s">
         <v>139</v>
@@ -3010,16 +3016,16 @@
         <v>48</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="N21" s="6" t="s">
         <v>53</v>
@@ -3034,7 +3040,7 @@
         <v>55</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="S21" s="6" t="s">
         <v>58</v>
@@ -3086,84 +3092,84 @@
         <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>115</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -3191,82 +3197,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -3297,19 +3303,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3320,13 +3326,13 @@
         <v>46308</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3337,30 +3343,30 @@
         <v>46319</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>224</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46333</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,13 +3377,13 @@
         <v>46310</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3415,13 +3421,13 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>36</v>
@@ -3442,10 +3448,10 @@
         <v>41</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3675,7 +3681,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUM(C2:C6)</f>
@@ -3716,7 +3722,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -3745,94 +3751,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22"/>
       <c r="B2" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22"/>
       <c r="B4" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22"/>
       <c r="B5" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Retarget Instagram plan to Saudi Arabia, Australia and New Zealand
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vRai2Js1dvdXXwRHYcreT
</commit_message>
<xml_diff>
--- a/marginwise/instagram-content-calendar.xlsx
+++ b/marginwise/instagram-content-calendar.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Setup before 14 Oct" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$Z$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$AA$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="266">
   <si>
     <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 15 Nov 2026</t>
   </si>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Rules</t>
   </si>
   <si>
-    <t xml:space="preserve">All posts go out at 19:30 IST. That is 10:00 US Eastern and 15:00 UK until the clocks change (UK 25 Oct, US 1 Nov); the Calendar tab shows the exact local times for each date.</t>
+    <t xml:space="preserve">From 18 Oct, posts for Australia, NZ or all markets go out at 13:30 IST (11:00 Riyadh, 19:00 Sydney, 21:00 Auckland). India and Saudi posts go out at 19:30 IST (17:00 Riyadh). The Calendar tab shows each date.</t>
   </si>
   <si>
     <t xml:space="preserve">No holiday greetings, memes or office posts. They underperformed for every competitor reviewed.</t>
@@ -91,10 +91,13 @@
     <t xml:space="preserve">IST</t>
   </si>
   <si>
-    <t xml:space="preserve">US Eastern</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UK</t>
+    <t xml:space="preserve">Riyadh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auckland</t>
   </si>
   <si>
     <t xml:space="preserve">Format</t>
@@ -163,10 +166,13 @@
     <t xml:space="preserve">19:30</t>
   </si>
   <si>
-    <t xml:space="preserve">10:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:00</t>
+    <t xml:space="preserve">17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03:00</t>
   </si>
   <si>
     <t xml:space="preserve">Reel (60s)</t>
@@ -175,7 +181,7 @@
     <t xml:space="preserve">Proof and trust</t>
   </si>
   <si>
-    <t xml:space="preserve">Both</t>
+    <t xml:space="preserve">All</t>
   </si>
   <si>
     <t xml:space="preserve">Every agency sells you ROAS. We sell you margin. This is what that looks like.</t>
@@ -291,7 +297,7 @@
     <t xml:space="preserve">COD/RTO</t>
   </si>
   <si>
-    <t xml:space="preserve">India</t>
+    <t xml:space="preserve">India + Saudi</t>
   </si>
   <si>
     <t xml:space="preserve">26% of your COD orders come back.</t>
@@ -322,13 +328,28 @@
     <t xml:space="preserve">Tue</t>
   </si>
   <si>
+    <t xml:space="preserve">13:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Teardown</t>
   </si>
   <si>
+    <t xml:space="preserve">ANZ</t>
+  </si>
+  <si>
     <t xml:space="preserve">[Brand] does everything right on this page except one thing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Screen-record a well-known US/UK brand's mobile product page. Two strengths, one leak (hidden shipping cost, review placement, or slow image). What that leak costs in margin.</t>
+    <t xml:space="preserve">Screen-record a well-known Australian or New Zealand brand's mobile product page. Two strengths, one leak (shipping cost hidden until checkout, Afterpay messaging buried, review placement, or a slow image). What that leak costs in margin.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Record: Phone screen-record (iOS Control Centre &gt; Screen Recording, or Android quick settings) the brand's mobile product page: scroll slowly, add to cart, open cart. 40 seconds, no notifications (Do Not Disturb on).
@@ -341,10 +362,13 @@
   <si>
     <t xml:space="preserve">A product page teardown with a margin lens: what converts, what leaks, and what the leak costs.
 Want this for your store? Comment AUDIT.
-#shopifycro #productpage #ecommerce</t>
+#shopifyaustralia #ecommerceaustralia #nzbusiness</t>
   </si>
   <si>
     <t xml:space="preserve">Thu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">India</t>
   </si>
   <si>
     <t xml:space="preserve">Your revenue is growing. Your profit isn't. Here's why.</t>
@@ -394,13 +418,10 @@
 #d2cindia #ecommerceindia #margin</t>
   </si>
   <si>
-    <t xml:space="preserve">14:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">Save these 5 checkout pages before you redesign yours.</t>
   </si>
   <si>
-    <t xml:space="preserve">Five public checkouts (mix of US/UK and Indian). One thing each does well: trust badges placement, delivery date, COD/prepaid nudge, express pay, order summary clarity.</t>
+    <t xml:space="preserve">Five public checkouts: two Australian or NZ, one Saudi, two Indian. One thing each does well: delivery date, express pay (Apple Pay, Afterpay, mada, UPI), COD/prepaid nudge, trust badges, order summary clarity.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Record: Phone screen-record five public checkouts (stop before payment). 6-8 seconds each.
@@ -469,10 +490,13 @@
     <t xml:space="preserve">Carousel (6 slides)</t>
   </si>
   <si>
-    <t xml:space="preserve">How a US or UK brand works with a team in India</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1 hook. S2 overlap hours (your morning, our evening). S3 weekly written update, with redacted example. S4 one senior contact. S5 billing in USD/GBP, NDA, 30-day notice. S6 CTA.</t>
+    <t xml:space="preserve">ANZ + Saudi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How Australian, NZ and Saudi brands work with a team in India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 overlap hours: Riyadh is 2.5 hours behind India, so the whole working day overlaps; Sydney and Auckland afternoons are India's morning. S3 weekly written update, with redacted example. S4 one senior contact. S5 billing in AUD, NZD or SAR, NDA, 30-day notice. S6 CTA.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
@@ -484,23 +508,23 @@
   </si>
   <si>
     <t xml:space="preserve">The three things founders worry about with an offshore team, and exactly how we handle each one.
-See how we work at the link in bio.
-#ecommerceagency #shopifyexperts #dtc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Link in bio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why US brands are scared to hire an agency in India.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Communication, time zones, quality. How each should be handled by any agency: overlap hours, weekly written update, one senior point of contact. 'Ask any agency for these three.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF scrolling to the 'If the agency is in another country' section, plus a world clock showing IST vs ET overlap.
+Comment CHECKLIST for the questions to ask any agency, us included.
+#ecommerceaustralia #saudibusiness #dtc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECKLIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marginwise-agency-checklist.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why founders worry about hiring an agency in India.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Communication, time zones, quality. How each should be handled by any agency: overlap hours (Riyadh shares India's working day; Sydney and Auckland afternoons are India's morning), weekly written update, one senior point of contact. 'Ask any agency for these three.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF scrolling to the 'If the agency is in another country' section, plus a world clock showing Riyadh, India, Sydney and Auckland side by side.
 2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Name the three worries, then the three answers.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
 4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text list builds one line at a time.
@@ -510,13 +534,7 @@
   <si>
     <t xml:space="preserve">What to ask any offshore agency before you sign, ourselves included.
 Comment CHECKLIST for the full agency hiring checklist.
-#ecommerceagency #shopify #dtcbrands</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHECKLIST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marginwise-agency-checklist.pdf</t>
+#ecommerceagency #shopifyaustralia #saudibusiness</t>
   </si>
   <si>
     <t xml:space="preserve">Retention</t>
@@ -572,10 +590,10 @@
     <t xml:space="preserve">marginwise-shopify-speed-checklist.pdf + speed check</t>
   </si>
   <si>
-    <t xml:space="preserve">Black Friday checkout checklist: 7 fixes before 27 November</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One fix per slide: shipping cost shown early, guest checkout, express pay, delivery date, stock and promo messaging, mobile speed, post-purchase upsell that keeps margin. Final slide CTA.</t>
+    <t xml:space="preserve">Sale-season checkout checklist: 7 fixes before Click Frenzy, White Friday and Black Friday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One fix per slide: shipping cost shown early, guest checkout, express pay (Apple Pay, Afterpay, mada, Tabby or Tamara), delivery date, honest offer messaging, mobile speed, post-purchase upsell that keeps margin. Final slide CTA.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
@@ -586,9 +604,9 @@
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Seven checkout fixes you can still ship before Black Friday, none of which need a redesign.
-Save this. Comment BFCM for the full checklist with a sale timeline.
-#blackfriday #bfcm #shopify</t>
+    <t xml:space="preserve">Seven checkout fixes you can still ship before the November sales, none of which need a redesign.
+Comment BFCM for the full checklist with a sale timeline.
+#blackfriday #clickfrenzy #whitefriday</t>
   </si>
   <si>
     <t xml:space="preserve">BFCM</t>
@@ -616,23 +634,23 @@
 #d2c #marketingagency #founders</t>
   </si>
   <si>
-    <t xml:space="preserve">Tariffs went up. Your prices didn't. Here's the gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Since the $800 de minimis exemption ended, landed costs rose. Landed cost before and after (illustrative). Three levers besides price: AOV bundles, free-shipping threshold, push higher-margin products.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator with COGS raised to show a tariff hit, then bundle/AOV changes recovering margin.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Before vs after landed cost; three levers.
+    <t xml:space="preserve">Buy now, pay later is not free. Here's what it costs you.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afterpay in Australia and NZ, Tabby and Tamara in Saudi: every BNPL order carries a merchant fee. Enter your own BNPL fee in the PROFIT calculator's payment fee line and show contribution per order before and after. Three levers: show BNPL only above a minimum order value, price bundles to lift AOV, steer repeat buyers to cheaper payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator: raise the payment fee line to your BNPL fee, then raise AOV to show margin recovering.
+2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Before vs after contribution per order; three levers.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
 4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Before/after numbers side by side as text.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rising import costs hit contribution margin first. Three ways to protect it without a price rise.
-Comment PROFIT for the margin calculator.
-#dtc #tariffs #shopify</t>
+    <t xml:space="preserve">BNPL can lift conversion, but every order pays a merchant fee. Know what it does to your margin before you push it.
+Comment PROFIT for the calculator and run it with your own fee.
+#afterpay #tabby #ecommerceaustralia</t>
   </si>
   <si>
     <t xml:space="preserve">Batch 3</t>
@@ -1624,33 +1642,33 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z21"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1732,6 +1750,9 @@
       <c r="Z1" s="5" t="s">
         <v>41</v>
       </c>
+      <c r="AA1" s="5" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
@@ -1741,63 +1762,66 @@
         <v>46309</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>50</v>
       </c>
+      <c r="K2" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="L2" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T2" s="9"/>
-      <c r="U2" s="10"/>
+        <v>59</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U2" s="9"/>
       <c r="V2" s="10"/>
       <c r="W2" s="10"/>
       <c r="X2" s="10"/>
       <c r="Y2" s="10"/>
       <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="n">
@@ -1807,63 +1831,66 @@
         <v>46311</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="S3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="6" t="s">
+      <c r="T3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T3" s="9"/>
-      <c r="U3" s="10"/>
+      <c r="U3" s="9"/>
       <c r="V3" s="10"/>
       <c r="W3" s="10"/>
       <c r="X3" s="10"/>
       <c r="Y3" s="10"/>
       <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="n">
@@ -1873,63 +1900,66 @@
         <v>46312</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>72</v>
+        <v>63</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T4" s="9"/>
-      <c r="U4" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U4" s="9"/>
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
       <c r="X4" s="10"/>
       <c r="Y4" s="10"/>
       <c r="Z4" s="10"/>
+      <c r="AA4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="n">
@@ -1939,63 +1969,66 @@
         <v>46313</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="J5" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>81</v>
       </c>
+      <c r="K5" s="8" t="s">
+        <v>82</v>
+      </c>
       <c r="L5" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T5" s="9"/>
-      <c r="U5" s="10"/>
+        <v>59</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U5" s="9"/>
       <c r="V5" s="10"/>
       <c r="W5" s="10"/>
       <c r="X5" s="10"/>
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
+      <c r="AA5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
@@ -2005,63 +2038,66 @@
         <v>46315</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>45</v>
+        <v>91</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>89</v>
+        <v>93</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>95</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P6" s="11" t="s">
         <v>56</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R6" s="11" t="s">
         <v>57</v>
       </c>
       <c r="S6" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T6" s="9"/>
-      <c r="U6" s="10"/>
+        <v>59</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U6" s="9"/>
       <c r="V6" s="10"/>
       <c r="W6" s="10"/>
       <c r="X6" s="10"/>
       <c r="Y6" s="10"/>
       <c r="Z6" s="10"/>
+      <c r="AA6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
@@ -2071,63 +2107,66 @@
         <v>46317</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J7" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>94</v>
+        <v>63</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>101</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="P7" s="11" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="Q7" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R7" s="11" t="s">
         <v>57</v>
       </c>
       <c r="S7" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T7" s="9"/>
-      <c r="U7" s="10"/>
+        <v>59</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U7" s="9"/>
       <c r="V7" s="10"/>
       <c r="W7" s="10"/>
       <c r="X7" s="10"/>
       <c r="Y7" s="10"/>
       <c r="Z7" s="10"/>
+      <c r="AA7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
@@ -2137,63 +2176,66 @@
         <v>46319</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J8" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="K8" s="11" t="s">
-        <v>101</v>
+      <c r="K8" s="13" t="s">
+        <v>108</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="Q8" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R8" s="11" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="S8" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T8" s="9"/>
-      <c r="U8" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U8" s="9"/>
       <c r="V8" s="10"/>
       <c r="W8" s="10"/>
       <c r="X8" s="10"/>
       <c r="Y8" s="10"/>
       <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
@@ -2203,63 +2245,66 @@
         <v>46320</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>106</v>
+        <v>93</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>112</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>53</v>
+        <v>115</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P9" s="11" t="s">
         <v>56</v>
       </c>
       <c r="Q9" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R9" s="11" t="s">
         <v>57</v>
       </c>
       <c r="S9" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T9" s="9"/>
-      <c r="U9" s="10"/>
+        <v>59</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U9" s="9"/>
       <c r="V9" s="10"/>
       <c r="W9" s="10"/>
       <c r="X9" s="10"/>
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
+      <c r="AA9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
@@ -2269,63 +2314,66 @@
         <v>46322</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G10" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="T10" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="N10" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="P10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="R10" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="S10" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T10" s="9"/>
-      <c r="U10" s="10"/>
+      <c r="U10" s="9"/>
       <c r="V10" s="10"/>
       <c r="W10" s="10"/>
       <c r="X10" s="10"/>
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
+      <c r="AA10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
@@ -2335,63 +2383,66 @@
         <v>46324</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>104</v>
+        <v>46</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>118</v>
+        <v>93</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>53</v>
+        <v>127</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P11" s="6" t="s">
         <v>56</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>116</v>
+        <v>57</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T11" s="9"/>
-      <c r="U11" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U11" s="9"/>
       <c r="V11" s="10"/>
       <c r="W11" s="10"/>
       <c r="X11" s="10"/>
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>
+      <c r="AA11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
@@ -2401,63 +2452,66 @@
         <v>46326</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>47</v>
+        <v>128</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>123</v>
+        <v>49</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>130</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T12" s="9"/>
-      <c r="U12" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U12" s="9"/>
       <c r="V12" s="10"/>
       <c r="W12" s="10"/>
       <c r="X12" s="10"/>
       <c r="Y12" s="10"/>
       <c r="Z12" s="10"/>
+      <c r="AA12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
@@ -2467,63 +2521,66 @@
         <v>46327</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="K13" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J13" s="6" t="s">
         <v>129</v>
       </c>
+      <c r="K13" s="8" t="s">
+        <v>136</v>
+      </c>
       <c r="L13" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>116</v>
+        <v>57</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T13" s="9"/>
-      <c r="U13" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U13" s="9"/>
       <c r="V13" s="10"/>
       <c r="W13" s="10"/>
       <c r="X13" s="10"/>
       <c r="Y13" s="10"/>
       <c r="Z13" s="10"/>
+      <c r="AA13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="n">
@@ -2533,63 +2590,66 @@
         <v>46329</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G14" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="P14" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q14" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R14" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="T14" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="K14" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="P14" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q14" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="R14" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="S14" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T14" s="9"/>
-      <c r="U14" s="10"/>
+      <c r="U14" s="9"/>
       <c r="V14" s="10"/>
       <c r="W14" s="10"/>
       <c r="X14" s="10"/>
       <c r="Y14" s="10"/>
       <c r="Z14" s="10"/>
+      <c r="AA14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
@@ -2599,63 +2659,66 @@
         <v>46331</v>
       </c>
       <c r="C15" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="G15" s="11" t="s">
+      <c r="H15" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="N15" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="P15" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q15" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="R15" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S15" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="T15" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="M15" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="N15" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="P15" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q15" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="R15" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="S15" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T15" s="9"/>
-      <c r="U15" s="10"/>
+      <c r="U15" s="9"/>
       <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="10"/>
       <c r="Z15" s="10"/>
+      <c r="AA15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
@@ -2665,63 +2728,66 @@
         <v>46333</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="J16" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>148</v>
+        <v>116</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="K16" s="13" t="s">
+        <v>153</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="P16" s="11" t="s">
-        <v>55</v>
+        <v>158</v>
       </c>
       <c r="Q16" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R16" s="11" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="S16" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T16" s="9"/>
-      <c r="U16" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="T16" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U16" s="9"/>
       <c r="V16" s="10"/>
       <c r="W16" s="10"/>
       <c r="X16" s="10"/>
       <c r="Y16" s="10"/>
       <c r="Z16" s="10"/>
+      <c r="AA16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
@@ -2731,63 +2797,66 @@
         <v>46334</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>104</v>
+        <v>46</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>154</v>
+        <v>49</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="K17" s="13" t="s">
+        <v>159</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>55</v>
+        <v>135</v>
       </c>
       <c r="Q17" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R17" s="11" t="s">
-        <v>116</v>
+        <v>57</v>
       </c>
       <c r="S17" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="T17" s="9"/>
-      <c r="U17" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="T17" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="U17" s="9"/>
       <c r="V17" s="10"/>
       <c r="W17" s="10"/>
       <c r="X17" s="10"/>
       <c r="Y17" s="10"/>
       <c r="Z17" s="10"/>
+      <c r="AA17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
@@ -2797,63 +2866,66 @@
         <v>46336</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>158</v>
+        <v>63</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>67</v>
+        <v>166</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>161</v>
+        <v>57</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T18" s="9"/>
-      <c r="U18" s="10"/>
+        <v>167</v>
+      </c>
+      <c r="T18" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U18" s="9"/>
       <c r="V18" s="10"/>
       <c r="W18" s="10"/>
       <c r="X18" s="10"/>
       <c r="Y18" s="10"/>
       <c r="Z18" s="10"/>
+      <c r="AA18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="n">
@@ -2863,63 +2935,66 @@
         <v>46338</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>104</v>
+        <v>46</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>162</v>
+        <v>47</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>61</v>
+        <v>168</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>164</v>
+        <v>63</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>169</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>97</v>
+        <v>172</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>161</v>
+        <v>57</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T19" s="9"/>
-      <c r="U19" s="10"/>
+        <v>167</v>
+      </c>
+      <c r="T19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U19" s="9"/>
       <c r="V19" s="10"/>
       <c r="W19" s="10"/>
       <c r="X19" s="10"/>
       <c r="Y19" s="10"/>
       <c r="Z19" s="10"/>
+      <c r="AA19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
@@ -2929,63 +3004,66 @@
         <v>46340</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>134</v>
+        <v>72</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>168</v>
+        <v>140</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>55</v>
+        <v>146</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T20" s="9"/>
-      <c r="U20" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="T20" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U20" s="9"/>
       <c r="V20" s="10"/>
       <c r="W20" s="10"/>
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
       <c r="Z20" s="10"/>
+      <c r="AA20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="n">
@@ -2995,68 +3073,71 @@
         <v>46341</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>172</v>
+        <v>49</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>53</v>
+        <v>180</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P21" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q21" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>161</v>
+        <v>57</v>
       </c>
       <c r="S21" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="T21" s="9"/>
-      <c r="U21" s="10"/>
+        <v>167</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="U21" s="9"/>
       <c r="V21" s="10"/>
       <c r="W21" s="10"/>
       <c r="X21" s="10"/>
       <c r="Y21" s="10"/>
       <c r="Z21" s="10"/>
+      <c r="AA21" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z21"/>
+  <autoFilter ref="A1:AA21"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="S2:S21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="T2:T21" type="list">
       <formula1>"Planned,Filmed,Edited,Scheduled,Posted,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3092,84 +3173,84 @@
         <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3197,82 +3278,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -3303,87 +3384,87 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46308</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46319</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46333</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>46310</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -3421,37 +3502,37 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3466,31 +3547,31 @@
         <v>4</v>
       </c>
       <c r="D2" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A2,Calendar!$S$2:$S$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A2,Calendar!$T$2:$T$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="F2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="G2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="H2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="I2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="J2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$AA$2:$AA$21)</f>
         <v>0</v>
       </c>
       <c r="K2" s="17" t="n">
@@ -3511,31 +3592,31 @@
         <v>4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A3,Calendar!$S$2:$S$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A3,Calendar!$T$2:$T$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="F3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="G3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="H3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="I3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="J3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$AA$2:$AA$21)</f>
         <v>0</v>
       </c>
       <c r="K3" s="17" t="n">
@@ -3556,31 +3637,31 @@
         <v>4</v>
       </c>
       <c r="D4" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A4,Calendar!$S$2:$S$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A4,Calendar!$T$2:$T$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="F4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="G4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="H4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="I4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="J4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$AA$2:$AA$21)</f>
         <v>0</v>
       </c>
       <c r="K4" s="17" t="n">
@@ -3601,31 +3682,31 @@
         <v>4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A5,Calendar!$S$2:$S$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A5,Calendar!$T$2:$T$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="F5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="G5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="H5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="I5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="J5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$AA$2:$AA$21)</f>
         <v>0</v>
       </c>
       <c r="K5" s="17" t="n">
@@ -3646,31 +3727,31 @@
         <v>4</v>
       </c>
       <c r="D6" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A6,Calendar!$S$2:$S$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A6,Calendar!$T$2:$T$21,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$U$2:$U$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$V$2:$V$21)</f>
         <v>0</v>
       </c>
       <c r="F6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$W$2:$W$21)</f>
         <v>0</v>
       </c>
       <c r="G6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$X$2:$X$21)</f>
         <v>0</v>
       </c>
       <c r="H6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Y$2:$Y$21)</f>
         <v>0</v>
       </c>
       <c r="I6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Z$2:$Z$21)</f>
         <v>0</v>
       </c>
       <c r="J6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$AA$2:$AA$21)</f>
         <v>0</v>
       </c>
       <c r="K6" s="17" t="n">
@@ -3681,7 +3762,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUM(C2:C6)</f>
@@ -3722,7 +3803,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3751,94 +3832,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22"/>
       <c r="B2" s="6" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22"/>
       <c r="B4" s="6" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22"/>
       <c r="B5" s="6" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="6" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refocus Instagram plan on Australia, US and UK with AI, SEO/AEO/GEO and web services
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vRai2Js1dvdXXwRHYcreT
</commit_message>
<xml_diff>
--- a/marginwise/instagram-content-calendar.xlsx
+++ b/marginwise/instagram-content-calendar.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="261">
   <si>
     <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 15 Nov 2026</t>
   </si>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Rules</t>
   </si>
   <si>
-    <t xml:space="preserve">From 18 Oct, posts for Australia, NZ or all markets go out at 13:30 IST (11:00 Riyadh, 19:00 Sydney, 21:00 Auckland). India and Saudi posts go out at 19:30 IST (17:00 Riyadh). The Calendar tab shows each date.</t>
+    <t xml:space="preserve">From 18 Oct the account targets Australia, the US and the UK. Australia posts go out at 13:30 IST (19:00 Sydney); US/UK and all-market posts at 19:30 IST (afternoon in London, morning in New York). The Calendar tab shows each date's local times.</t>
   </si>
   <si>
     <t xml:space="preserve">No holiday greetings, memes or office posts. They underperformed for every competitor reviewed.</t>
@@ -91,13 +91,13 @@
     <t xml:space="preserve">IST</t>
   </si>
   <si>
-    <t xml:space="preserve">Riyadh</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sydney</t>
   </si>
   <si>
-    <t xml:space="preserve">Auckland</t>
+    <t xml:space="preserve">London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New York</t>
   </si>
   <si>
     <t xml:space="preserve">Format</t>
@@ -166,13 +166,13 @@
     <t xml:space="preserve">19:30</t>
   </si>
   <si>
-    <t xml:space="preserve">17:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">01:00</t>
   </si>
   <si>
-    <t xml:space="preserve">03:00</t>
+    <t xml:space="preserve">15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:00</t>
   </si>
   <si>
     <t xml:space="preserve">Reel (60s)</t>
@@ -191,7 +191,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. Record: Screen-record (desktop, QuickTime or OBS, 1080p) a walkthrough of an audit on a demo store: GA4 funnel, three leaks marked in a doc, the one-page written summary. Use a Shopify dev store or public pages only.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Open with: 'This is what we look at before we touch your ads.'
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Open with: 'This is what we look at before we touch your ads.'
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
 4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Zoom (keyframes) on each leak as you name it; red box highlights. Pin this post after publishing.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
@@ -242,7 +242,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator (ROAS to Profit tab) at 150% zoom, typing in a 3x ROAS store and watching contribution turn negative.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Say each cost as it is subtracted; end on the break-even ROAS cell.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Say each cost as it is subtracted; end on the break-even ROAS cell.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
 4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the cell being changed each time; end frame on the verdict cell.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
@@ -291,38 +291,36 @@
     <t xml:space="preserve">Sun</t>
   </si>
   <si>
-    <t xml:space="preserve">Reel (50s)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COD/RTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">India + Saudi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26% of your COD orders come back.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shipway FY25: 26% RTO on COD vs under 2% prepaid. What one RTO costs: forward and return shipping, packaging, wasted ad spend. Three fixes: prepaid incentive, WhatsApp confirmation for risky COD, switch off COD only in high-RTO pin codes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the RTO finder with sample orders loaded: the By State tab sorting by cost, one state flagged 'Restrict COD or verify'.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Use the Shipway 26% vs under 2% figure in the first line.
+    <t xml:space="preserve">Reel (10s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO/AEO/GEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We asked ChatGPT to recommend a brand in your category. Were you in the answer?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record asking ChatGPT, Perplexity and Google (AI Overview) the same buying question for one category, for example 'best running socks in Australia'. Show which brands get named and which don't. Takeaway: AI search is a new shelf, and you can work on getting onto it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record (desktop) ChatGPT, Perplexity and Google with the same buying question; scroll the answers slowly.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Open: 'We asked AI what to buy.' End on 'Comment GEO'.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text callout for each of the three fixes as you say it.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight each brand name the AI mentions; blur nothing needed, these are public answers.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Switching off COD everywhere is the wrong fix. Find the pin codes where it loses money and act only there.
-Comment RTO and we will send you the sheet that ranks your states and pin codes by RTO cost.
-#d2cindia #rto #shopifyindia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marginwise-rto-finder.xlsx + marginwise-cod-rto-playbook.pdf</t>
+    <t xml:space="preserve">Shoppers now ask ChatGPT, Perplexity and Google's AI answers what to buy. Some brands get named. Most don't.
+Getting into those answers is a mix of SEO, clear product pages and being mentioned in the right places.
+Comment GEO and we will send you the AI search visibility checklist.
+#aisearch #seo #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marginwise-ai-search-visibility-checklist.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Tue</t>
@@ -331,103 +329,102 @@
     <t xml:space="preserve">13:30</t>
   </si>
   <si>
-    <t xml:space="preserve">11:00</t>
-  </si>
-  <si>
     <t xml:space="preserve">19:00</t>
   </si>
   <si>
-    <t xml:space="preserve">21:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teardown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANZ</t>
+    <t xml:space="preserve">09:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AU</t>
   </si>
   <si>
     <t xml:space="preserve">[Brand] does everything right on this page except one thing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Screen-record a well-known Australian or New Zealand brand's mobile product page. Two strengths, one leak (shipping cost hidden until checkout, Afterpay messaging buried, review placement, or a slow image). What that leak costs in margin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Phone screen-record (iOS Control Centre &gt; Screen Recording, or Android quick settings) the brand's mobile product page: scroll slowly, add to cart, open cart. 40 seconds, no notifications (Do Not Disturb on).
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Two things it does well, then the one leak and what it costs.
+    <t xml:space="preserve">Phone screen-record a well-known Australian brand's mobile product page. Two strengths, one leak (shipping cost hidden until checkout, Afterpay message buried, reviews too low, or a slow image). What that leak costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record the Australian brand's mobile product page: scroll, add to cart, open cart. Do Not Disturb on.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Two things it does well, then the one leak and what it costs.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red circle on the leak; slow-zoom into it. Blur any personal data.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red circle on the leak; slow zoom.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">A product page teardown with a margin lens: what converts, what leaks, and what the leak costs.
+    <t xml:space="preserve">A product page teardown of an Australian brand: what converts, what leaks, and what the leak costs.
 Want this for your store? Comment AUDIT.
-#shopifyaustralia #ecommerceaustralia #nzbusiness</t>
+#shopifyaustralia #ecommerceaustralia #cro</t>
   </si>
   <si>
     <t xml:space="preserve">Thu</t>
   </si>
   <si>
-    <t xml:space="preserve">India</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your revenue is growing. Your profit isn't. Here's why.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Break down a ₹1,000 order: GST, COGS, ad cost per order, shipping, RTO, gateway fees, discounts. Land on contribution margin per order. Investors now ask for this, not GMV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the MARGIN calculator, Margin per Order tab, stepping through each cost line of a ₹1,000 order.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. One sentence per cost line; end on contribution per order.
+    <t xml:space="preserve">Performance marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US/UK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before you raise your Meta budget, check these 3 numbers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the PROFIT calculator. 1) Break-even ROAS, 2) contribution per order after ads, 3) new vs returning customer share in Shopify. If any is off, more budget scales the loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator at 150% zoom, then Shopify's new vs returning customer report (demo store).
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. One sentence per number; end on 'more budget scales the loss'.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Running total as on-screen text in the top corner.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight each number as you name it.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Contribution margin per order, explained with a real ₹1,000 example.
-Comment MARGIN and we will send you the calculator, including a what-if for pushing more buyers to prepaid.
-#d2cindia #unitEconomics #founders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARGIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marginwise-margin-calculator-inr.xlsx + marginwise-contribution-margin-checklist.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carousel (8 slides)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What a ₹1,000 order actually earns you</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One cost per slide: GST, product cost, ad cost, shipping and packaging, RTO, COD fees, gateway fees. Final slide: contribution per order and the one lever that moves it most.</t>
+    <t xml:space="preserve">More budget does not fix a campaign that loses money on every order. It scales it.
+Check break-even ROAS, contribution after ads and your new-customer share first.
+Comment PROFIT for the calculator.
+#metaads #performancemarketing #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to show up when shoppers ask AI what to buy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 AI answers pull from pages they can read: check your robots.txt and site speed. S3 product pages that answer real questions (sizing, materials, delivery, returns). S4 structured data: Product, Offer, Review and FAQ schema. S5 reviews and mentions on other sites, not only your own. S6 test it monthly: ask ChatGPT, Perplexity and Google the same 5 buying questions and log who appears. S7 CTA.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
-2. Slide copy: take it from the Outline column. Max 25 words per slide. One cost per slide with the running total shown on every slide.
+2. Slide copy: take it from the Outline column. Max 25 words per slide. Same template as the first carousel. Check every claim against its source line.
 3. Put a source line (small, bottom) on every slide with a statistic.
 4. Last slide: CTA with the comment keyword in large text.
 5. Export as PNG, upload in order, add alt text to slide 1.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Line by line, what is left of a ₹1,000 order once every cost is counted. Numbers are an example store; run your own with the calculator.
-Comment MARGIN for the sheet.
-#d2cindia #ecommerceindia #margin</t>
+    <t xml:space="preserve">SEO still matters. AI search adds a second test: can an AI answer engine read your pages, trust them and quote them?
+Five things you control, and a simple monthly test.
+Comment GEO for the full checklist.
+#aeo #geo #seo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:00</t>
   </si>
   <si>
     <t xml:space="preserve">Save these 5 checkout pages before you redesign yours.</t>
   </si>
   <si>
-    <t xml:space="preserve">Five public checkouts: two Australian or NZ, one Saudi, two Indian. One thing each does well: delivery date, express pay (Apple Pay, Afterpay, mada, UPI), COD/prepaid nudge, trust badges, order summary clarity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Phone screen-record five public checkouts (stop before payment). 6-8 seconds each.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. One line per checkout: what it does well.
+    <t xml:space="preserve">Phone screen-record five public checkouts from US, UK and Australian brands. One thing each does well: delivery date, express pay (Shop Pay, Apple Pay, Afterpay, Klarna), guest checkout, trust near the pay button, order summary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record five public checkouts (US, UK, AU); stop before payment. 2 seconds each.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. One line per checkout: what it does well.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Numbered label 1-5 on screen; 'Save this' text on the final frame.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Numbered labels 1-5; 'Save this' on the final frame.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
@@ -437,121 +434,111 @@
 #checkout #shopify #cro</t>
   </si>
   <si>
-    <t xml:space="preserve">CRO</t>
-  </si>
-  <si>
     <t xml:space="preserve">7 out of 10 people who add to cart never buy.</t>
   </si>
   <si>
-    <t xml:space="preserve">Baymard: 70.22% average cart abandonment across 50 studies. Three fixable reasons: surprise costs, forced account creation, too many steps. Show one fix for each on a Shopify checkout.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Phone screen-record a checkout showing a surprise shipping cost, a forced account screen and a long form (public stores).
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Lead with Baymard's 70.22%; one fix per problem.
+    <t xml:space="preserve">Baymard: 70.22% average cart abandonment across 50 studies. Three fixable reasons: surprise costs, forced account creation, too many steps. One fix for each on a Shopify checkout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record a checkout with a surprise shipping cost, a forced account screen and a long form (public stores).
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Lead with Baymard's 70.22%; one fix per problem.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Split screen: problem on top, fix described as text below.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Problem on top, fix as text below.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Cart abandonment averages 70% (Baymard Institute). Three fixes that do not need a redesign.
-Save this for your next checkout review.
+Comment AUDIT for the 30-point store leak audit.
 #checkout #shopifytips #ecommerce</t>
   </si>
   <si>
-    <t xml:space="preserve">Save</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
     <t xml:space="preserve">Batch 2</t>
   </si>
   <si>
-    <t xml:space="preserve">[Indian Brand] is losing mobile buyers here.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screen-record an Indian D2C brand's mobile product page. Two strengths, one leak (COD/prepaid messaging, delivery date clarity, size guidance). The fix.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Phone screen-record the Indian brand's mobile product page: price, delivery date, COD/prepaid messaging, size guide.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Two strengths, one leak, the fix.
+    <t xml:space="preserve">AI solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is what an AI support assistant for a Shopify store looks like.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record a demo on a Shopify development store: a shopper asks 'where is my order' and 'can I return this', the assistant answers from store policies and order status, and hands over to a person when it is unsure. Demo store only, no client data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a support assistant demo on a Shopify development store (Shopify Inbox, or the tool you use). Demo data only.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Two shopper questions, the answers, then the hand-over to a person.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red circle on the leak; ₹ figures as on-screen text.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text callouts: 'answers from your policies', 'hands over when unsure'.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most support tickets are the same five questions. An AI assistant can answer them in seconds, from your own policies, and pass anything unusual to your team.
+Comment AI for 10 AI builds worth starting with for ecommerce brands.
+#aiforbusiness #shopify #ecommerce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marginwise-ai-for-ecommerce-builds.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousel (6 slides)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How US, UK and Australian brands work with a team in India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 overlap hours: London afternoons and US mornings are India's evening; Sydney evenings are India's afternoon. S3 weekly written update, with a redacted example. S4 one senior contact. S5 billing in USD, GBP or AUD, NDA, 30-day notice. S6 CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The three things founders worry about with an offshore team, and exactly how we handle each one.
+Comment CHECKLIST for the questions to ask any agency, us included.
+#ecommerceagency #shopifyexperts #dtc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECKLIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marginwise-agency-checklist.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How we use AI in a store audit, and what we never hand to it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record: AI summarises 500 product reviews into the top objections, drafts test ideas and writes the first pass of the report. Then show what a person does: checks the data, decides priorities, writes the recommendation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record an AI tool summarising public reviews of a demo product, then your audit doc where you set priorities.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. What AI does, then what a person does.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Split screen: 'AI' on top, 'Person' below.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">A mobile product page teardown of an Indian D2C brand, and one fix that lifts conversion without a redesign.
-Comment AUDIT for a teardown of your store.
-#d2cindia #cro #shopifyindia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carousel (6 slides)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANZ + Saudi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How Australian, NZ and Saudi brands work with a team in India</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1 hook. S2 overlap hours: Riyadh is 2.5 hours behind India, so the whole working day overlaps; Sydney and Auckland afternoons are India's morning. S3 weekly written update, with redacted example. S4 one senior contact. S5 billing in AUD, NZD or SAR, NDA, 30-day notice. S6 CTA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
-2. Slide copy: take it from the Outline column. Max 25 words per slide. Slide 3 shows a redacted sample weekly update; build it from a blank template, not client data.
-3. Put a source line (small, bottom) on every slide with a statistic.
-4. Last slide: CTA with the comment keyword in large text.
-5. Export as PNG, upload in order, add alt text to slide 1.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The three things founders worry about with an offshore team, and exactly how we handle each one.
-Comment CHECKLIST for the questions to ask any agency, us included.
-#ecommerceaustralia #saudibusiness #dtc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHECKLIST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marginwise-agency-checklist.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why founders worry about hiring an agency in India.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Communication, time zones, quality. How each should be handled by any agency: overlap hours (Riyadh shares India's working day; Sydney and Auckland afternoons are India's morning), weekly written update, one senior point of contact. 'Ask any agency for these three.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF scrolling to the 'If the agency is in another country' section, plus a world clock showing Riyadh, India, Sydney and Auckland side by side.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Name the three worries, then the three answers.
+    <t xml:space="preserve">AI makes our audits faster: it reads every review, drafts test ideas and does the first pass of the report.
+It does not decide what to fix first. A person who has built D2C products does that.
+Comment AUDIT for a free 2-minute teardown of your store.
+#ai #cro #ecommerce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating post-purchase emails. This one is a 2/10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screenshot three order confirmation emails (your own inbox, details blurred). Score each with one reason; end on what a 9/10 contains.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screenshot three order confirmation emails from your own inbox; blur names, order numbers and addresses.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Score each out of 10 with one reason.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Text list builds one line at a time.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Big score number on each email.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What to ask any offshore agency before you sign, ourselves included.
-Comment CHECKLIST for the full agency hiring checklist.
-#ecommerceagency #shopifyaustralia #saudibusiness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rating post-purchase emails. This one is a 2/10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate three order confirmation emails (public or redacted) with a score and one reason each. End on what a 9/10 email contains.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screenshot three order confirmation emails (your own inbox; blur names, order numbers, addresses).
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Score each out of 10 with one reason; end on what a 9/10 has.
-3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Big score number appears on each email; slow scroll down each one.
-5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Your order confirmation email is the most-opened email you send. Most brands waste it on a receipt.
@@ -565,23 +552,26 @@
     <t xml:space="preserve">marginwise-post-purchase-email-checklist.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">Website development</t>
+  </si>
+  <si>
     <t xml:space="preserve">A tenth of a second changed conversions by 8.4%.</t>
   </si>
   <si>
-    <t xml:space="preserve">Deloitte/Google study of 37 brands. Run a public store through PageSpeed. Show the three usual culprits: app scripts, oversized images, third-party widgets. Fix speed before buying more traffic.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record pagespeed.web.dev running on a public Shopify store, then the opportunities list.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Lead with Deloitte/Google 0.1s = 8.4%; name the three culprits.
+    <t xml:space="preserve">Deloitte/Google study of 37 brands. Run a public store through PageSpeed and show the three usual culprits: app scripts, oversized images, third-party widgets. Fix speed before buying more traffic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record pagespeed.web.dev on a public Shopify store, then the opportunities list.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Lead with 0.1s = 8.4%; name the three culprits.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the three culprits in the report as you name them.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the three culprits as you name them.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">Fix speed before you buy more traffic. The three culprits on most Shopify stores.
 Comment SPEED and we will check your store.
-#shopifyspeed #cro #ecommerce</t>
+#shopifyspeed #webdevelopment #cro</t>
   </si>
   <si>
     <t xml:space="preserve">SPEED</t>
@@ -590,23 +580,18 @@
     <t xml:space="preserve">marginwise-shopify-speed-checklist.pdf + speed check</t>
   </si>
   <si>
-    <t xml:space="preserve">Sale-season checkout checklist: 7 fixes before Click Frenzy, White Friday and Black Friday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One fix per slide: shipping cost shown early, guest checkout, express pay (Apple Pay, Afterpay, mada, Tabby or Tamara), delivery date, honest offer messaging, mobile speed, post-purchase upsell that keeps margin. Final slide CTA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
-2. Slide copy: take it from the Outline column. Max 25 words per slide. One fix per slide with a small mock of the checkout element it refers to.
-3. Put a source line (small, bottom) on every slide with a statistic.
-4. Last slide: CTA with the comment keyword in large text.
-5. Export as PNG, upload in order, add alt text to slide 1.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seven checkout fixes you can still ship before the November sales, none of which need a redesign.
+    <t xml:space="preserve">Carousel (8 slides)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Friday checklist: 7 checkout fixes before 27 November</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One fix per slide: shipping cost shown early, guest checkout, express pay (Shop Pay, Apple Pay, Afterpay, Klarna), delivery date, honest offer messaging, mobile speed, post-purchase upsell that keeps margin. Final slide CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seven checkout fixes you can still ship before Black Friday and Click Frenzy, none of which need a redesign.
 Comment BFCM for the full checklist with a sale timeline.
-#blackfriday #clickfrenzy #whitefriday</t>
+#blackfriday #bfcm #clickfrenzy</t>
   </si>
   <si>
     <t xml:space="preserve">BFCM</t>
@@ -615,105 +600,95 @@
     <t xml:space="preserve">marginwise-black-friday-checklist.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">Five questions to ask before you hire a D2C agency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Who works on my account? Whose name is the ad account in? Show a redacted report with CPA. Notice period? Which one metric in month one?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the agency checklist PDF, top table (five questions, good answer, red flag).
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Read each question and its red flag.
+    <t xml:space="preserve">Theme, custom build or headless? Most stores pick the wrong one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record three stores side by side. Theme: fastest and cheapest, fine for most stores under a certain size. Custom Shopify build: when the brand or the funnel needs it. Headless: when you have the team to maintain it. One question to decide: who will maintain it next year?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record three public stores: one on a standard theme, one custom, one headless.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. One line per option and who it suits; end on the maintenance question.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight each row as you read it.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Labels: Theme, Custom, Headless.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Most founders pick an agency from the pitch deck. Ask these five questions instead, including to us.
-Comment CHECKLIST for the full list.
-#d2c #marketingagency #founders</t>
+    <t xml:space="preserve">A new website is a business decision, not a design one. Pick the build you can afford to maintain.
+Comment AUDIT and we will tell you which one your store needs.
+#shopify #webdevelopment #headless</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch 3</t>
   </si>
   <si>
     <t xml:space="preserve">Buy now, pay later is not free. Here's what it costs you.</t>
   </si>
   <si>
-    <t xml:space="preserve">Afterpay in Australia and NZ, Tabby and Tamara in Saudi: every BNPL order carries a merchant fee. Enter your own BNPL fee in the PROFIT calculator's payment fee line and show contribution per order before and after. Three levers: show BNPL only above a minimum order value, price bundles to lift AOV, steer repeat buyers to cheaper payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator: raise the payment fee line to your BNPL fee, then raise AOV to show margin recovering.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Before vs after contribution per order; three levers.
+    <t xml:space="preserve">Afterpay, Klarna, Clearpay and Affirm all charge a merchant fee on every order. Enter your own BNPL fee in the PROFIT calculator's payment fee line and show contribution per order before and after. Three levers: show BNPL above a minimum order value, bundle to lift AOV, steer repeat buyers to cheaper payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator: raise the payment fee to your BNPL fee, then raise AOV to recover margin.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Before vs after contribution per order; three levers.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Before/after numbers side by side as text.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Before/after numbers side by side.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
     <t xml:space="preserve">BNPL can lift conversion, but every order pays a merchant fee. Know what it does to your margin before you push it.
 Comment PROFIT for the calculator and run it with your own fee.
-#afterpay #tabby #ecommerceaustralia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batch 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reel (40s)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your ₹1 lakh ad budget costs ₹1.18 lakh.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta Ireland billing means 18% GST under reverse charge, paid in cash before credit. Show the cash timing. Add 18% to the ad budget in your cash-flow plan. Confirm with your CA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record the MARGIN calculator, GST on Ads tab, typing ₹1,00,000.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Explain reverse charge in one sentence; say 'confirm with your CA'.
+#afterpay #klarna #ecommerce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI-written product descriptions: 3 rules so they sell, rank and get cited.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record an AI tool drafting a product description from a spec sheet, then edit it live: 1) add the facts shoppers ask about (size, material, care, delivery), 2) write for the questions people search, 3) a person checks every claim before it goes live.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record an AI tool drafting a product description for a demo product, then your edits in the Shopify editor.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. The three rules, one per edit.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Show '₹1,18,000 leaves your account' as the final frame.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Strike-through on generic lines, highlight on added facts.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">The GST line that catches founders short on cash. Not tax advice; confirm with your CA.
-Comment MARGIN for the calculator, which includes a GST-on-ads tab.
-#d2cindia #metaads #gst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After the sale: turn festive and Black Friday buyers into repeat buyers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1 hook. S2 why sale buyers churn. S3 the delivered + how-to-use email. S4 review request timing. S5 replenishment timed to your data. S6 win-back without a discount first. S7 CTA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Canva &gt; Instagram Post (portrait) 1080x1350. Use one template for every carousel: navy background, white text, one idea per slide.
-2. Slide copy: take it from the Outline column. Max 25 words per slide. Each email slide shows when to send it and one line of example copy.
-3. Put a source line (small, bottom) on every slide with a statistic.
-4. Last slide: CTA with the comment keyword in large text.
-5. Export as PNG, upload in order, add alt text to slide 1.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+    <t xml:space="preserve">AI can write 500 product descriptions in an hour. Without rules, they all sound the same and answer nothing.
+Three rules we use so they sell, rank in search and get quoted by AI answers.
+Comment AI for 10 AI builds worth starting with.
+#ai #seo #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After Black Friday: turn sale buyers into repeat buyers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 why sale buyers churn. S3 the delivered and how-to-use email. S4 review request timing. S5 replenishment timed to your data. S6 win-back without a discount first. S7 CTA.</t>
   </si>
   <si>
     <t xml:space="preserve">Sale buyers are the easiest to lose. Five emails that bring them back without giving away margin.
 Comment FLOWS for the full checklist.
-#retention #emailmarketing #d2c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">We audited [N] D2C stores this month. The same 3 leaks showed up in [X] of them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only post if the audits are real; use the actual count. Three most common leaks, anonymised. If fewer than 5 audits are done, swap for a second Indian teardown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record a tally sheet of the audits you actually ran (store names hidden) and anonymised screenshots of the three leaks.
-2. Script the voiceover (about 130 words for 60s): hook, the work, the takeaway, CTA. Use the real count. If under 5 audits, swap for a second Indian teardown and follow that recipe.
+#retention #emailmarketing #dtc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We audited [N] stores this month. The same 3 leaks showed up in [X] of them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only post if the audits are real; use the actual count. Three most common leaks, anonymised. If fewer than 5 audits are done, swap for a second Australian teardown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a tally of audits you actually ran (store names hidden) and anonymised screenshots of the three leaks.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Use the real count; if under 5, record a second Australian teardown instead.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Counter animation for each leak's tally.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Counter for each leak's tally.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">What we keep finding when we audit D2C stores, with no names attached.
+    <t xml:space="preserve">What we keep finding when we audit ecommerce stores, with no names attached.
 Comment AUDIT to get yours.
-#d2c #cro #ecommercegrowth</t>
+#ecommerce #cro #shopify</t>
   </si>
   <si>
     <t xml:space="preserve">Story type</t>
@@ -779,6 +754,9 @@
     <t xml:space="preserve">Answer one question from DMs as 2-3 text frames over a screen recording or screenshot of the relevant page.</t>
   </si>
   <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
     <t xml:space="preserve">Turns DMs into content and shows you reply.</t>
   </si>
   <si>
@@ -821,7 +799,7 @@
     <t xml:space="preserve">Editing</t>
   </si>
   <si>
-    <t xml:space="preserve">CapCut: 9:16, Auto captions, hook text in the first 2 seconds, cut every pause over half a second, zoom and red-box highlights on whatever you name. Length 30-60 seconds.</t>
+    <t xml:space="preserve">CapCut: 9:16, Auto captions, hook text in the first 2 seconds, cut every pause over half a second, zoom and red-box highlights on whatever you name. Length 10 seconds; Google Flow clips work as b-roll.</t>
   </si>
   <si>
     <t xml:space="preserve">Privacy</t>
@@ -857,37 +835,34 @@
     <t xml:space="preserve">Time needed</t>
   </si>
   <si>
-    <t xml:space="preserve">Founder intro; ROAS 3x; COD RTO 26%; US/UK product page teardown; ₹1,000 order margin; 5 checkout pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pick the US/UK brand and 5 checkouts (public pages). Record all screen captures first, then write and record every voiceover in one sitting.</t>
+    <t xml:space="preserve">AI search test (GEO); Australian product page teardown; Meta budget numbers; 5 checkouts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick the category question for the AI test, the Australian brand and five public checkouts. Record screens first, then all voiceovers in one sitting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cart abandonment; AI support assistant demo; how we use AI in an audit; email ratings; site speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set up the Shopify development store with demo products and policies for the AI demos.</t>
   </si>
   <si>
     <t xml:space="preserve">3 hours</t>
   </si>
   <si>
-    <t xml:space="preserve">Cart abandonment; Indian teardown; offshore trust; email ratings; site speed; agency questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pick the Indian brand and three order confirmation emails (your own inbox or public examples). Run PageSpeed on one public store.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tariffs; GST on ads; audit roundup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count real audits done so far. If fewer than 5, film a second Indian teardown instead of the roundup.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 hours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All five carousels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use the same template: navy and white, one idea per slide, source line on every stat slide. Canva or Figma.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 hours</t>
+    <t xml:space="preserve">Theme vs custom vs headless; BNPL fees; AI product descriptions; audit roundup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count the real audits done so far. If fewer than 5, record a second Australian teardown instead of the roundup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousels: AI search visibility, offshore trust, Black Friday checklist, after-the-sale retention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same template as the first carousel: navy, white text, green numbers, one idea per slide.</t>
   </si>
   <si>
     <t xml:space="preserve">Week starting</t>
@@ -935,7 +910,7 @@
     <t xml:space="preserve">A hacked brand account is hard to recover</t>
   </si>
   <si>
-    <t xml:space="preserve">All lead magnets (3 sheets, 8 PDFs) uploaded to Drive or the website with share links</t>
+    <t xml:space="preserve">All lead magnets (1 sheet, 8 PDFs) uploaded to Drive or the website with share links</t>
   </si>
   <si>
     <t xml:space="preserve">Every CTA keyword depends on these</t>
@@ -965,7 +940,7 @@
     <t xml:space="preserve">Before posting anything publicly</t>
   </si>
   <si>
-    <t xml:space="preserve">UK decision made (keep in bio and site, or remove)</t>
+    <t xml:space="preserve">Website updated for Australia, US and UK (hours, currency, services)</t>
   </si>
   <si>
     <t xml:space="preserve">Bio and website must match</t>
@@ -1990,25 +1965,25 @@
         <v>80</v>
       </c>
       <c r="J5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="L5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="M5" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="N5" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="O5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="P5" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="Q5" s="6" t="s">
         <v>58</v>
@@ -2038,40 +2013,40 @@
         <v>46315</v>
       </c>
       <c r="C6" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="F6" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="G6" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="H6" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="H6" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="11" t="s">
+      <c r="J6" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="K6" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="L6" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="M6" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="N6" s="11" t="s">
         <v>97</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>98</v>
       </c>
       <c r="O6" s="11" t="s">
         <v>55</v>
@@ -2107,7 +2082,7 @@
         <v>46317</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>44</v>
@@ -2122,10 +2097,10 @@
         <v>47</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>100</v>
@@ -2143,10 +2118,10 @@
         <v>104</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="P7" s="11" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="Q7" s="11" t="s">
         <v>57</v>
@@ -2191,31 +2166,31 @@
         <v>47</v>
       </c>
       <c r="H8" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K8" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="M8" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="K8" s="13" t="s">
+      <c r="N8" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="L8" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>111</v>
-      </c>
       <c r="O8" s="11" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="Q8" s="11" t="s">
         <v>57</v>
@@ -2248,37 +2223,37 @@
         <v>78</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="G9" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>92</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>93</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K9" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="M9" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>55</v>
@@ -2314,46 +2289,46 @@
         <v>46322</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="G10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="M10" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="J10" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="K10" s="8" t="s">
+      <c r="N10" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="L10" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="N10" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="O10" s="6" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="Q10" s="6" t="s">
         <v>58</v>
@@ -2362,7 +2337,7 @@
         <v>57</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T10" s="6" t="s">
         <v>60</v>
@@ -2383,7 +2358,7 @@
         <v>46324</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>44</v>
@@ -2392,37 +2367,37 @@
         <v>45</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>47</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K11" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="O11" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="P11" s="6" t="s">
         <v>125</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="P11" s="6" t="s">
-        <v>56</v>
       </c>
       <c r="Q11" s="6" t="s">
         <v>58</v>
@@ -2431,7 +2406,7 @@
         <v>57</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T11" s="6" t="s">
         <v>60</v>
@@ -2455,43 +2430,43 @@
         <v>71</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>49</v>
       </c>
       <c r="J12" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="N12" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="O12" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="P12" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="Q12" s="6" t="s">
         <v>57</v>
@@ -2524,43 +2499,43 @@
         <v>78</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>49</v>
+        <v>119</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>129</v>
+        <v>50</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>135</v>
+        <v>56</v>
       </c>
       <c r="Q13" s="6" t="s">
         <v>57</v>
@@ -2569,7 +2544,7 @@
         <v>57</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T13" s="6" t="s">
         <v>60</v>
@@ -2590,46 +2565,46 @@
         <v>46329</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E14" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>92</v>
-      </c>
       <c r="H14" s="11" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J14" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K14" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="O14" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="P14" s="11" t="s">
         <v>142</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="P14" s="11" t="s">
-        <v>146</v>
       </c>
       <c r="Q14" s="11" t="s">
         <v>58</v>
@@ -2638,7 +2613,7 @@
         <v>57</v>
       </c>
       <c r="S14" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T14" s="11" t="s">
         <v>60</v>
@@ -2659,46 +2634,46 @@
         <v>46331</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G15" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>92</v>
-      </c>
       <c r="H15" s="11" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="J15" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K15" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="N15" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="O15" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="M15" s="11" t="s">
+      <c r="P15" s="11" t="s">
         <v>149</v>
-      </c>
-      <c r="N15" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="P15" s="11" t="s">
-        <v>152</v>
       </c>
       <c r="Q15" s="11" t="s">
         <v>57</v>
@@ -2707,7 +2682,7 @@
         <v>57</v>
       </c>
       <c r="S15" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="T15" s="11" t="s">
         <v>60</v>
@@ -2731,43 +2706,43 @@
         <v>71</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" s="11" t="s">
+      <c r="H16" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="J16" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K16" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="M16" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="I16" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="K16" s="13" t="s">
+      <c r="N16" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="L16" s="11" t="s">
+      <c r="O16" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="M16" s="11" t="s">
+      <c r="P16" s="11" t="s">
         <v>155</v>
-      </c>
-      <c r="N16" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="O16" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="P16" s="11" t="s">
-        <v>158</v>
       </c>
       <c r="Q16" s="11" t="s">
         <v>57</v>
@@ -2806,37 +2781,37 @@
         <v>45</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="J17" s="11" t="s">
         <v>100</v>
       </c>
       <c r="K17" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="N17" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="L17" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="M17" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>162</v>
-      </c>
       <c r="O17" s="11" t="s">
-        <v>134</v>
+        <v>55</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>135</v>
+        <v>56</v>
       </c>
       <c r="Q17" s="11" t="s">
         <v>57</v>
@@ -2845,7 +2820,7 @@
         <v>57</v>
       </c>
       <c r="S17" s="11" t="s">
-        <v>123</v>
+        <v>160</v>
       </c>
       <c r="T17" s="11" t="s">
         <v>60</v>
@@ -2866,40 +2841,40 @@
         <v>46336</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>129</v>
+        <v>50</v>
       </c>
       <c r="K18" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="M18" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="L18" s="6" t="s">
+      <c r="N18" s="6" t="s">
         <v>164</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>166</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>69</v>
@@ -2914,7 +2889,7 @@
         <v>57</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="T18" s="6" t="s">
         <v>60</v>
@@ -2935,7 +2910,7 @@
         <v>46338</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>44</v>
@@ -2944,37 +2919,37 @@
         <v>45</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>168</v>
+        <v>79</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>100</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="Q19" s="6" t="s">
         <v>57</v>
@@ -2983,7 +2958,7 @@
         <v>57</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="T19" s="6" t="s">
         <v>60</v>
@@ -3007,43 +2982,43 @@
         <v>71</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>72</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>50</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>175</v>
+        <v>107</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="Q20" s="6" t="s">
         <v>57</v>
@@ -3076,19 +3051,19 @@
         <v>78</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>92</v>
-      </c>
       <c r="H21" s="6" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>49</v>
@@ -3097,16 +3072,16 @@
         <v>50</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="O21" s="6" t="s">
         <v>55</v>
@@ -3121,7 +3096,7 @@
         <v>57</v>
       </c>
       <c r="S21" s="6" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="T21" s="6" t="s">
         <v>60</v>
@@ -3173,84 +3148,84 @@
         <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>122</v>
+        <v>197</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -3278,82 +3253,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3384,19 +3359,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>223</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3404,50 +3379,50 @@
         <v>59</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>46308</v>
+        <v>46313</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46319</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B4" s="7" t="n">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3455,16 +3430,16 @@
         <v>77</v>
       </c>
       <c r="B5" s="7" t="n">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3502,13 +3477,13 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>37</v>
@@ -3529,10 +3504,10 @@
         <v>42</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,7 +3737,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUM(C2:C6)</f>
@@ -3803,7 +3778,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3832,94 +3807,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22"/>
       <c r="B2" s="6" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22"/>
       <c r="B4" s="6" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22"/>
       <c r="B5" s="6" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="6" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="6" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Instagram calendar to 13 Dec: research-led posts, Germany and Canada, solution demos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vRai2Js1dvdXXwRHYcreT
</commit_message>
<xml_diff>
--- a/marginwise/instagram-content-calendar.xlsx
+++ b/marginwise/instagram-content-calendar.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Setup before 14 Oct" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$AA$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calendar!$A$1:$AA$37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,12 +29,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="261">
-  <si>
-    <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 15 Nov 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Five weeks, 20 posts: 3 reels and 1 carousel a week, plus Stories on 4 days. Built from marginwise/instagram-playbook.md.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="342">
+  <si>
+    <t xml:space="preserve">Marginwise Instagram content calendar: 14 Oct to 13 Dec 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nine weeks, 36 posts: about 3 reels and 1 carousel a week, plus Stories on 4 days. Built from marginwise/instagram-playbook.md and the market research of 17 Oct 2026. Weeks 1-5: Australia, US and UK. Weeks 6-9 add Germany (Berlin, English) and Canada. Saudi Arabia starts in the next calendar. Germany posts go out at 19:30 IST, which is London time plus one hour in Berlin; Canada follows New York.</t>
   </si>
   <si>
     <t xml:space="preserve">Tabs</t>
@@ -220,7 +220,7 @@
     <t xml:space="preserve">Batch 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Planned</t>
+    <t xml:space="preserve">Posted</t>
   </si>
   <si>
     <t xml:space="preserve">Fri</t>
@@ -323,6 +323,9 @@
     <t xml:space="preserve">marginwise-ai-search-visibility-checklist.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">Planned</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tue</t>
   </si>
   <si>
@@ -347,7 +350,7 @@
     <t xml:space="preserve">[Brand] does everything right on this page except one thing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Phone screen-record a well-known Australian brand's mobile product page. Two strengths, one leak (shipping cost hidden until checkout, Afterpay message buried, reviews too low, or a slow image). What that leak costs.</t>
+    <t xml:space="preserve">Phone screen-record a well-known Australian brand's mobile product page. Two strengths, one leak (card surcharge still showing after the 1 Oct ban, shipping cost hidden until checkout, Afterpay message buried, reviews too low, or a slow image). What that leak costs. Set the store to Australia and A$ before recording.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Record: Phone screen-record the Australian brand's mobile product page: scroll, add to cart, open cart. Do Not Disturb on.
@@ -434,23 +437,27 @@
 #checkout #shopify #cro</t>
   </si>
   <si>
-    <t xml:space="preserve">7 out of 10 people who add to cart never buy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baymard: 70.22% average cart abandonment across 50 studies. Three fixable reasons: surprise costs, forced account creation, too many steps. One fix for each on a Shopify checkout.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Phone screen-record a checkout with a surprise shipping cost, a forced account screen and a long form (public stores).
-2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Lead with Baymard's 70.22%; one fix per problem.
+    <t xml:space="preserve">08:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since 1 October, this line is banned in Australian checkouts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone screen-record a checkout (demo store) showing a '1.5% card surcharge' line, then the same checkout without it. The RBA ban on surcharging Visa, Mastercard and eftpos started 1 Oct 2026. Two things follow: the line must go, and the fee lands in your margin unless prices or payment mix change. Show a payment-fee margin table with one SKU in red.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record the demo store checkout with a '1.5% card surcharge' line, then without it; then the payment-fee margin table.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Open on the ban date; end on 'who pays the fee now?'.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Problem on top, fix as text below.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Red strike-through on the surcharge line; one SKU row highlighted red.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cart abandonment averages 70% (Baymard Institute). Three fixes that do not need a redesign.
-Comment AUDIT for the 30-point store leak audit.
-#checkout #shopifytips #ecommerce</t>
+    <t xml:space="preserve">The RBA ban on card surcharges started on 1 October. If your checkout still adds a card fee, it has to go.
+Then the real question: who pays the fee now? Absorb it, reprice, or steer customers to cheaper ways to pay.
+Comment PROFIT for the calculator and run your own card fees through it.
+#ecommerceaustralia #shopifyaustralia #payments</t>
   </si>
   <si>
     <t xml:space="preserve">Batch 2</t>
@@ -504,24 +511,24 @@
     <t xml:space="preserve">marginwise-agency-checklist.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">How we use AI in a store audit, and what we never hand to it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screen-record: AI summarises 500 product reviews into the top objections, drafts test ideas and writes the first pass of the report. Then show what a person does: checks the data, decides priorities, writes the recommendation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record an AI tool summarising public reviews of a demo product, then your audit doc where you set priorities.
-2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. What AI does, then what a person does.
+    <t xml:space="preserve">We built a tool that audits a store in two minutes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the Marginwise audit crawler running on the demo store (terminal command, then the report): score out of 100, red rows for speed, trackers firing before consent, missing product schema, and one market rule (AU surcharge or German Impressum). End: a person checks every finding before it goes to you.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the terminal running the audit crawler on the demo store, then scroll the HTML report.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Tool first, person second: 'a person checks every finding'.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Split screen: 'AI' on top, 'Person' below.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Zoom on the score, then on three red rows.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI makes our audits faster: it reads every review, drafts test ideas and does the first pass of the report.
-It does not decide what to fix first. A person who has built D2C products does that.
-Comment AUDIT for a free 2-minute teardown of your store.
-#ai #cro #ecommerce</t>
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every free teardown starts with our audit tool: speed, accessibility, tracking, checkout, local rules and AI search readiness, scored in two minutes.
+Then a person checks every finding and picks the one fix that matters most.
+Comment AUDIT and we will run it on your store.
+#ai #cro #shopify</t>
   </si>
   <si>
     <t xml:space="preserve">Retention</t>
@@ -600,23 +607,27 @@
     <t xml:space="preserve">marginwise-black-friday-checklist.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">Theme, custom build or headless? Most stores pick the wrong one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screen-record three stores side by side. Theme: fastest and cheapest, fine for most stores under a certain size. Custom Shopify build: when the brand or the funnel needs it. Headless: when you have the team to maintain it. One question to decide: who will maintain it next year?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record three public stores: one on a standard theme, one custom, one headless.
-2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. One line per option and who it suits; end on the maintenance question.
+    <t xml:space="preserve">US</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four tariff changes in twelve months. Is your price still right?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record a landed-cost table for 5 demo SKUs: product cost, duty, tariff surcharge, freight, then margin. Change the tariff input and watch two SKUs turn red. Point: price on today's landed cost, not last quarter's. No legal or customs advice; rates come from your broker.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a landed-cost sheet for 5 demo SKUs; change the tariff input live.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Lead with 'four changes in a year'; end on 'price on today's landed cost'.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Labels: Theme, Custom, Headless.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Two SKUs flip to red; on-screen note 'rates from your broker'.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
 6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
   </si>
   <si>
-    <t xml:space="preserve">A new website is a business decision, not a design one. Pick the build you can afford to maintain.
-Comment AUDIT and we will tell you which one your store needs.
-#shopify #webdevelopment #headless</t>
+    <t xml:space="preserve">De minimis is gone and tariffs changed four times in a year. Most brands are still pricing on an old landed cost.
+Run your SKUs through today's numbers before Black Friday discounts eat what is left.
+Comment PROFIT for the calculator.
+#tariffs #ecommerce #shopify</t>
   </si>
   <si>
     <t xml:space="preserve">Batch 3</t>
@@ -641,24 +652,24 @@
 #afterpay #klarna #ecommerce</t>
   </si>
   <si>
-    <t xml:space="preserve">AI-written product descriptions: 3 rules so they sell, rank and get cited.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screen-record an AI tool drafting a product description from a spec sheet, then edit it live: 1) add the facts shoppers ask about (size, material, care, delivery), 2) write for the questions people search, 3) a person checks every claim before it goes live.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Record: Screen-record an AI tool drafting a product description for a demo product, then your edits in the Shopify editor.
-2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. The three rules, one per edit.
+    <t xml:space="preserve">Every morning, someone fixes these by hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the sync exception agent demo (fixture data): a list of failed Shopify-to-ERP orders, the agent labelling each cause (missing SKU, duplicate, tax code), safe fixes retried, two waiting for approval, then a 7am Slack summary '12 fixed, 2 need you'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the sync exception agent demo output (fixture data) and a mock Slack message.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Problem, what the agent does, what still needs a person.
 3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
-4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Strike-through on generic lines, highlight on added facts.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Labels on each error type; '12 fixed, 2 need you' as the end frame.
 5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
-6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI can write 500 product descriptions in an hour. Without rules, they all sound the same and answer nothing.
-Three rules we use so they sell, rank in search and get quoted by AI answers.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If your Shopify orders fail to reach Cin7, NetSuite, Xero or MYOB, someone is fixing them by hand every morning.
+An AI agent can sort the failures, fix the safe ones and leave the rest for a person to approve.
 Comment AI for 10 AI builds worth starting with.
-#ai #seo #shopify</t>
+#ai #shopify #erp</t>
   </si>
   <si>
     <t xml:space="preserve">After Black Friday: turn sale buyers into repeat buyers</t>
@@ -691,6 +702,311 @@
 #ecommerce #cro #shopify</t>
   </si>
   <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selling to Germany? Since 19 June your shop needs this button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone screen-record a German shop's footer and account area looking for the withdrawal button (Widerrufsbutton), then the two-step withdrawal flow on the demo store. Mention: public pages only, no shop named, and your lawyer confirms the wording.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record a German shop footer and account area (public, unnamed), then the demo store's two-step withdrawal flow.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Date first (19 June), then the fix; say 'your lawyer confirms the wording'.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Circle where the button should be; blur the shop's logo.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since 19 June 2026, online shops selling to German consumers need a withdrawal button: a two-step way to cancel a purchase during the withdrawal period.
+Missing it is an easy target for warning letters. Your lawyer confirms the wording; we build it into the theme.
+Comment AUDIT and we will check your shop.
+#ecommercegermany #shopify #berlinstartups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipping to the US from Canada? Your customer might be paying at the door.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record a demo checkout for a US customer from a Canadian store: no duties shown, then a mock delivery notice with brokerage and duty owed. Then the same checkout with duties-included pricing. Mention de minimis is gone and tariffs rose on many Canadian goods; your broker confirms rates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a US checkout on the demo store without duties, a mock delivery notice, then the duties-included version.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. The surprise at the door, then the fix; 'your broker confirms rates'.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Mock notice clearly labelled 'example'.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With de minimis gone, US customers of Canadian stores can be hit with duties and brokerage at the door. Many never order again.
+Duties-included pricing fixes the surprise, and shows you which SKUs still make money.
+Comment PROFIT for the calculator.
+#shopifycanada #ecommercecanada #crossborder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Friday week: 5 checks for the night before</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 place a test order on mobile with each payment method. S3 check discount codes and automatic discounts stack the way you planned. S4 shipping cut-off dates shown on product and cart pages. S5 tracking fires once per order (no double purchases in GA4 or Meta). S6 someone on DMs and email on the day. S7 CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Five checks to run the night before Black Friday, Click Frenzy or Cyber Monday. None of them need a developer.
+Save this for next week. Comment BFCM for the full checklist and timeline.
+#blackfriday #bfcm #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your store on Black Friday: test these 3 pages before the traffic does.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record PageSpeed (mobile) on the demo store's home, collection and product pages, then an app list showing two unused apps still loading scripts. Fix: remove them before the sale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record PageSpeed mobile on three demo store pages and the installed apps list.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Three pages, one culprit, one fix.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Score numbers large on screen.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic spikes expose slow pages. Test home, collection and product pages on mobile this week, and remove apps you no longer use.
+Comment SPEED and we will check your store before the sale.
+#shopifyspeed #blackfriday #cro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is why month-end takes three days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the payout reconciliation demo (fixture data): Shopify, PayPal and Afterpay payouts next to the bank feed, nothing lines up; the matcher runs, 412 of 418 matched with fees and refunds split out; the six exceptions explained in plain English. Demo data only, labelled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the payout reconciliation demo: inputs side by side, the match result, the exceptions summary.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Pain, result, what is left.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Counter '412 / 418 matched'; label 'demo data'.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopify Payments, PayPal, Afterpay and Klarna payouts rarely match the bank feed line for line. That is why month-end drags.
+We match every payout to the bank and explain what is left in plain English.
+Comment AI for 10 AI builds worth starting with.
+#xero #shopify #ecommercefinance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thanksgiving orders are in. Send this email before the box arrives.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screenshot an order confirmation and a 'your order is on its way' email from your own inbox (details blurred). Show one change: tell the customer how to use the product and when to expect it, not just a receipt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screenshot two order emails from your own inbox, blurred; mock up the improved version in Canva.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Before and after; one change.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Before/after split.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The emails after a Black Friday order decide whether that customer buys again in January.
+Start with the order confirmation and the shipping email.
+Comment FLOWS for the post-purchase checklist.
+#klaviyo #bfcm #emailmarketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It's Black Friday. Three fixes you can still ship in an hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone screen-record three quick fixes on the demo store: free-shipping threshold shown in the cart, express pay buttons above the fold in checkout, and a delivery cut-off banner. 3 seconds each.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Phone screen-record three quick changes on the demo store.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. One line per fix; 'no developer needed'.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Numbered labels 1-3.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three changes you can still make today without a developer: show the free-shipping threshold in the cart, put express pay first, and add a delivery cut-off banner.
+Comment BFCM for the full checklist.
+#blackfriday #bfcm #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From 1 January 2027, a PDF invoice is not enough in Germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 who: businesses above EUR 800K turnover must issue B2B e-invoices from 1 Jan 2027, all businesses from 2028. S3 what counts: XRechnung or ZUGFeRD; a plain PDF does not. S4 where Shopify stores get stuck: no native DATEV link, B2B orders mixed with B2C. S5 what to set up: invoice output, DATEV export, payout matching. S6 confirm the rules with your tax adviser. S7 CTA. Source line: German Finance Ministry letter of 15 Oct 2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany's B2B e-invoicing rules start biting on 1 January 2027. If you sell to businesses from a Shopify or Shopware store, a PDF invoice will no longer count.
+Your tax adviser confirms what applies to you; we build the invoice output and the DATEV export.
+Comment AUDIT and tell us your setup.
+#erechnung #ecommercegermany #shopify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyber Monday is over. Read these 4 numbers before you celebrate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the PROFIT calculator with demo BFCM numbers: revenue up, but discount depth, returns allowance, ad cost and payment fees take contribution per order down. Four numbers: contribution per order, new-customer share, discount depth, returns rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the PROFIT calculator with demo BFCM numbers.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Revenue up, contribution down; the four numbers.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight each number as you name it.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Record revenue does not mean record profit. Before you celebrate, check contribution per order, new-customer share, discount depth and returns.
+Comment PROFIT for the calculator.
+#cybermonday #bfcm #ecommerce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google now charges some businesses for calls they miss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the AI receptionist demo: a missed call at 9:47pm, a text-back within a minute, then the AI answering a second call, saying it is an AI, checking the suburb and booking a job into a demo calendar. Mention Google Local Services Ads started billing for missed calls on 1 Oct 2026. Demo line only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the receptionist demo: phone missed-call screen, text-back, call transcript, demo calendar.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Lead with the Google change; the AI says it is an AI.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Time stamp '9:47pm' on screen; 'demo line' label.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since 1 October, Google bills Local Services Ads advertisers for missed calls during business hours. Every missed call now costs twice.
+An AI receptionist answers, says it is an AI, books the job and texts back the calls you miss.
+Comment AI to see it on a test line.
+#smallbusiness #hvac #ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selling into Quebec: what Bill 96 changes for your store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 French must be available to Quebec customers on your storefront and product information. S3 since 1 June 2025, generic words on packaging also need French; grace period to 1 June 2027 for older stock. S4 Law 25: consent before non-essential cookies. S5 what to do: French storefront with human-reviewed translation, consent banner, packaging to your lawyer. S6 CTA. Not legal advice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quebec has its own rules for language and privacy. If you sell there, check your storefront, your product data and your cookie banner.
+Packaging and legal wording go to your lawyer; we build the French store and the consent setup.
+Comment AUDIT and we will check your store.
+#quebec #shopifycanada #ecommercecanada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three page changes that make AI assistants quote your store.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the demo store's product page before and after: answers to real questions on the page (sizing, materials, delivery, returns), Product and FAQ schema validated in Google's Rich Results Test, and robots.txt allowing AI crawlers. No claims about ranking results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the demo product page before and after, Rich Results Test, and robots.txt.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Three changes, one per shot.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Tick on each change.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI assistants quote pages they can read and trust. Three changes help: answer real questions on the page, add Product and FAQ schema, and let AI crawlers in.
+Comment GEO for the full checklist.
+#aeo #geo #seo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Klimaneutral' is now a risky word on German product pages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the compliance copy auditor demo on fixture copy: a product page with a 'klimaneutral' badge, the finding (rule, risk, suggested rewrite), and a lawyer sign-off column. Rules since 27 Sep 2026 limit offset-based climate claims and self-made labels. Not legal advice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the compliance copy auditor output on fixture copy.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Date, the risky word, the safer rewrite, lawyer signs off.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Highlight the flagged phrase and the rewrite.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST as a Trial Reel (share to followers only if 3-second hold beats your average). Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since 27 September, claims like 'klimaneutral' based on offsetting and self-made eco labels are a risk in Germany.
+We scan your product pages and ads, flag each claim with a safer rewrite, and your lawyer signs off.
+Comment AUDIT and we will scan your shop.
+#greenclaims #ecommercegermany #berlinstartups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas orders plus Cin7 equals oversells. Here's the 7am fix.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen-record the sync exception agent demo again, framed for Christmas peak: stock mismatch errors, the agent flagging oversell risk and holding those SKUs for approval, then the Slack summary. Demo data only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record the sync agent demo with stock-mismatch fixtures and the Slack summary.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Peak season framing; what the agent holds for approval.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. 'Held for approval' label on the risky SKUs.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak season is when Shopify and your inventory system disagree most, and every mismatch is an oversell waiting to happen.
+An AI agent watches the sync, fixes what is safe and flags the rest before the morning rush.
+Comment AI for 10 AI builds worth starting with.
+#shopifyaustralia #cin7 #ecommerceaustralia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What changed for online stores in 2026, by country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1 hook. S2 Australia: card surcharge ban (1 Oct), subscription and drip-pricing rules from 1 Jul 2027. S3 US: de minimis gone, tariff changes, accessibility lawsuits. S4 UK: keep this slide general unless a rule is checked before posting. S5 Germany: withdrawal button (19 Jun), green claims (27 Sep), e-invoicing (1 Jan 2027). S6 Canada: Quebec French and cookie consent. S7 CTA. Source line on every slide; not legal advice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The rules for online stores changed a lot this year. One slide per country, with the date each change starts.
+Save this for your 2027 planning. Comment AUDIT and we will check your store against them.
+#ecommerce #shopify #compliance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What we found auditing stores this quarter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only post with real numbers: the count of audits run since October and the three most common findings, anonymised. If fewer than 5 audits are done, swap for a teardown of a German or Canadian store instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Record: Screen-record a tally of real audits (store names hidden) and anonymised screenshots of the top three findings.
+2. Script the voiceover (about 25 words for 10 seconds): hook, the work, the CTA. Use the real count; if under 5 audits, record a German or Canadian teardown instead.
+3. Voiceover: record in a quiet room on your phone (Voice Memos or CapCut &gt; Audio &gt; Record). One clean take; no AI voice.
+4. Edit in CapCut (9:16): drop in recordings, lay voiceover, Auto captions on (white, bold, lower third), hook text on screen for the first 2 seconds. Counter for each finding.
+5. Cover: freeze a frame of the work with the hook text on it; keep text inside the centre 1080x1080 so it crops cleanly on the grid.
+6. Post: paste caption from this sheet, add the location-free cover, turn on the auto-DM keyword, publish at 19:30 IST. Reply to every comment in the first hour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The leaks we found most often this quarter, with no names attached.
+Comment AUDIT to get yours checked before January.
+#ecommerce #cro #shopify</t>
+  </si>
+  <si>
     <t xml:space="preserve">Story type</t>
   </si>
   <si>
@@ -844,25 +1160,55 @@
     <t xml:space="preserve">2 hours</t>
   </si>
   <si>
-    <t xml:space="preserve">Cart abandonment; AI support assistant demo; how we use AI in an audit; email ratings; site speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set up the Shopify development store with demo products and policies for the AI demos.</t>
+    <t xml:space="preserve">Carousels: AI search visibility, offshore trust, Black Friday checklist, after-the-sale retention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same template as the first carousel: navy, white text, green numbers, one idea per slide.</t>
   </si>
   <si>
     <t xml:space="preserve">3 hours</t>
   </si>
   <si>
-    <t xml:space="preserve">Theme vs custom vs headless; BNPL fees; AI product descriptions; audit roundup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count the real audits done so far. If fewer than 5, record a second Australian teardown instead of the roundup.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carousels: AI search visibility, offshore trust, Black Friday checklist, after-the-sale retention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same template as the first carousel: navy, white text, green numbers, one idea per slide.</t>
+    <t xml:space="preserve">AU surcharge ban; AI support assistant demo; audit crawler demo; email ratings; site speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set up the Shopify development store with demo products, policies and a surcharge line to remove. Run the audit crawler on it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US tariffs and landed cost; BNPL fees; ERP sync agent demo; audit roundup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepare 5 demo SKUs for the landed-cost sheet. Run the sync exception agent on its fixtures.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany withdrawal button; Canada duties at the door; Black Friday page speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find one public German shop (unnamed in the post) and set up a US checkout on the demo store.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payout reconciliation demo; Thanksgiving email; Black Friday quick fixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the payout reconciliation agent on its fixtures; screenshot two order emails.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyber Monday numbers; AI receptionist demo; AI search page changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set up a demo phone line for the receptionist (or record from fixtures). Add schema to the demo product page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">German green claims; Christmas oversells; quarter roundup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run the compliance copy auditor and sync agent on fixtures. Count the real audits done.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carousels: Black Friday night-before checks, German e-invoicing, Quebec Bill 96, 2026 rules by country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same template as earlier carousels. Every rule slide gets a date and a source line; mark 'not legal advice'.</t>
   </si>
   <si>
     <t xml:space="preserve">Week starting</t>
@@ -922,7 +1268,7 @@
     <t xml:space="preserve">Broken DMs waste the first reels</t>
   </si>
   <si>
-    <t xml:space="preserve">Highlight covers made: Teardowns, How we work, US/UK clients, COD/RTO, Book a call</t>
+    <t xml:space="preserve">Highlight covers made: Teardowns, How we work, Tools we built, Book a call</t>
   </si>
   <si>
     <t xml:space="preserve">Profile looks complete from day one</t>
@@ -1526,7 +1872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1617,7 +1963,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AA37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1995,7 +2341,7 @@
         <v>59</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U5" s="9"/>
       <c r="V5" s="10"/>
@@ -2013,40 +2359,40 @@
         <v>46315</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O6" s="11" t="s">
         <v>55</v>
@@ -2064,7 +2410,7 @@
         <v>59</v>
       </c>
       <c r="T6" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U6" s="9"/>
       <c r="V6" s="10"/>
@@ -2082,7 +2428,7 @@
         <v>46317</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>44</v>
@@ -2100,22 +2446,22 @@
         <v>79</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O7" s="11" t="s">
         <v>69</v>
@@ -2133,7 +2479,7 @@
         <v>59</v>
       </c>
       <c r="T7" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U7" s="9"/>
       <c r="V7" s="10"/>
@@ -2175,16 +2521,16 @@
         <v>50</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O8" s="11" t="s">
         <v>85</v>
@@ -2202,7 +2548,7 @@
         <v>77</v>
       </c>
       <c r="T8" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U8" s="9"/>
       <c r="V8" s="10"/>
@@ -2229,7 +2575,7 @@
         <v>45</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>47</v>
@@ -2238,22 +2584,22 @@
         <v>79</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="O9" s="11" t="s">
         <v>55</v>
@@ -2271,7 +2617,7 @@
         <v>59</v>
       </c>
       <c r="T9" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U9" s="9"/>
       <c r="V9" s="10"/>
@@ -2289,46 +2635,46 @@
         <v>46322</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="Q10" s="6" t="s">
         <v>58</v>
@@ -2337,10 +2683,10 @@
         <v>57</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U10" s="9"/>
       <c r="V10" s="10"/>
@@ -2358,7 +2704,7 @@
         <v>46324</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>44</v>
@@ -2367,7 +2713,7 @@
         <v>45</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>47</v>
@@ -2376,28 +2722,28 @@
         <v>79</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>50</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="Q11" s="6" t="s">
         <v>58</v>
@@ -2406,10 +2752,10 @@
         <v>57</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U11" s="9"/>
       <c r="V11" s="10"/>
@@ -2436,13 +2782,13 @@
         <v>45</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>47</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>49</v>
@@ -2451,22 +2797,22 @@
         <v>50</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="Q12" s="6" t="s">
         <v>57</v>
@@ -2478,7 +2824,7 @@
         <v>77</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U12" s="9"/>
       <c r="V12" s="10"/>
@@ -2505,31 +2851,31 @@
         <v>45</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>50</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>55</v>
@@ -2538,16 +2884,16 @@
         <v>56</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U13" s="9"/>
       <c r="V13" s="10"/>
@@ -2565,7 +2911,7 @@
         <v>46329</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>44</v>
@@ -2574,37 +2920,37 @@
         <v>45</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H14" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J14" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="M14" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q14" s="11" t="s">
         <v>58</v>
@@ -2613,10 +2959,10 @@
         <v>57</v>
       </c>
       <c r="S14" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T14" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U14" s="9"/>
       <c r="V14" s="10"/>
@@ -2634,7 +2980,7 @@
         <v>46331</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>44</v>
@@ -2643,37 +2989,37 @@
         <v>45</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J15" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="Q15" s="11" t="s">
         <v>57</v>
@@ -2682,10 +3028,10 @@
         <v>57</v>
       </c>
       <c r="S15" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="T15" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U15" s="9"/>
       <c r="V15" s="10"/>
@@ -2712,37 +3058,37 @@
         <v>45</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J16" s="11" t="s">
         <v>50</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P16" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="Q16" s="11" t="s">
         <v>57</v>
@@ -2754,7 +3100,7 @@
         <v>77</v>
       </c>
       <c r="T16" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U16" s="9"/>
       <c r="V16" s="10"/>
@@ -2781,37 +3127,37 @@
         <v>45</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>79</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>143</v>
+        <v>100</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="Q17" s="11" t="s">
         <v>57</v>
@@ -2820,10 +3166,10 @@
         <v>57</v>
       </c>
       <c r="S17" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="T17" s="11" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U17" s="9"/>
       <c r="V17" s="10"/>
@@ -2841,7 +3187,7 @@
         <v>46336</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>44</v>
@@ -2850,31 +3196,31 @@
         <v>45</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>50</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>69</v>
@@ -2889,10 +3235,10 @@
         <v>57</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U18" s="9"/>
       <c r="V18" s="10"/>
@@ -2910,7 +3256,7 @@
         <v>46338</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>44</v>
@@ -2919,49 +3265,49 @@
         <v>45</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>79</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R19" s="6" t="s">
         <v>57</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U19" s="9"/>
       <c r="V19" s="10"/>
@@ -2988,37 +3334,37 @@
         <v>45</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>72</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>50</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q20" s="6" t="s">
         <v>57</v>
@@ -3030,7 +3376,7 @@
         <v>77</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U20" s="9"/>
       <c r="V20" s="10"/>
@@ -3057,10 +3403,10 @@
         <v>45</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>79</v>
@@ -3072,16 +3418,16 @@
         <v>50</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="O21" s="6" t="s">
         <v>55</v>
@@ -3096,10 +3442,10 @@
         <v>57</v>
       </c>
       <c r="S21" s="6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="U21" s="9"/>
       <c r="V21" s="10"/>
@@ -3109,10 +3455,1114 @@
       <c r="Z21" s="10"/>
       <c r="AA21" s="10"/>
     </row>
+    <row r="22" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>46343</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="J22" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="N22" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="O22" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="P22" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q22" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R22" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S22" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="T22" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U22" s="9"/>
+      <c r="V22" s="10"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="10"/>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="10"/>
+    </row>
+    <row r="23" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>46345</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="J23" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="N23" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="O23" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="P23" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q23" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S23" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="T23" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U23" s="9"/>
+      <c r="V23" s="10"/>
+      <c r="W23" s="10"/>
+      <c r="X23" s="10"/>
+      <c r="Y23" s="10"/>
+      <c r="Z23" s="10"/>
+      <c r="AA23" s="10"/>
+    </row>
+    <row r="24" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>46347</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="J24" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="N24" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="O24" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="P24" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q24" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="R24" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S24" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="T24" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U24" s="9"/>
+      <c r="V24" s="10"/>
+      <c r="W24" s="10"/>
+      <c r="X24" s="10"/>
+      <c r="Y24" s="10"/>
+      <c r="Z24" s="10"/>
+      <c r="AA24" s="10"/>
+    </row>
+    <row r="25" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>46348</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="N25" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="O25" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="P25" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q25" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="R25" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S25" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="T25" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U25" s="9"/>
+      <c r="V25" s="10"/>
+      <c r="W25" s="10"/>
+      <c r="X25" s="10"/>
+      <c r="Y25" s="10"/>
+      <c r="Z25" s="10"/>
+      <c r="AA25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>46350</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K26" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="M26" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="N26" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="O26" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="P26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q26" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="R26" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S26" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="T26" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U26" s="9"/>
+      <c r="V26" s="10"/>
+      <c r="W26" s="10"/>
+      <c r="X26" s="10"/>
+      <c r="Y26" s="10"/>
+      <c r="Z26" s="10"/>
+      <c r="AA26" s="10"/>
+    </row>
+    <row r="27" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>46352</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="M27" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="O27" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="P27" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q27" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R27" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S27" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="T27" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U27" s="9"/>
+      <c r="V27" s="10"/>
+      <c r="W27" s="10"/>
+      <c r="X27" s="10"/>
+      <c r="Y27" s="10"/>
+      <c r="Z27" s="10"/>
+      <c r="AA27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>46353</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="M28" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="N28" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S28" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="T28" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U28" s="9"/>
+      <c r="V28" s="10"/>
+      <c r="W28" s="10"/>
+      <c r="X28" s="10"/>
+      <c r="Y28" s="10"/>
+      <c r="Z28" s="10"/>
+      <c r="AA28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>46355</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="M29" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="N29" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="O29" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P29" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q29" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R29" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S29" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="T29" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U29" s="9"/>
+      <c r="V29" s="10"/>
+      <c r="W29" s="10"/>
+      <c r="X29" s="10"/>
+      <c r="Y29" s="10"/>
+      <c r="Z29" s="10"/>
+      <c r="AA29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K30" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="M30" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="N30" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="O30" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="P30" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q30" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R30" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S30" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="T30" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U30" s="9"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="X30" s="10"/>
+      <c r="Y30" s="10"/>
+      <c r="Z30" s="10"/>
+      <c r="AA30" s="10"/>
+    </row>
+    <row r="31" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>46359</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="M31" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="N31" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="O31" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="P31" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q31" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="R31" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S31" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="T31" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U31" s="9"/>
+      <c r="V31" s="10"/>
+      <c r="W31" s="10"/>
+      <c r="X31" s="10"/>
+      <c r="Y31" s="10"/>
+      <c r="Z31" s="10"/>
+      <c r="AA31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>46361</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="J32" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="K32" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="N32" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="O32" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="P32" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q32" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="R32" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S32" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="T32" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U32" s="9"/>
+      <c r="V32" s="10"/>
+      <c r="W32" s="10"/>
+      <c r="X32" s="10"/>
+      <c r="Y32" s="10"/>
+      <c r="Z32" s="10"/>
+      <c r="AA32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>46362</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K33" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="O33" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="P33" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q33" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="R33" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="S33" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="T33" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="U33" s="9"/>
+      <c r="V33" s="10"/>
+      <c r="W33" s="10"/>
+      <c r="X33" s="10"/>
+      <c r="Y33" s="10"/>
+      <c r="Z33" s="10"/>
+      <c r="AA33" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>46364</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P34" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q34" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S34" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="T34" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U34" s="9"/>
+      <c r="V34" s="10"/>
+      <c r="W34" s="10"/>
+      <c r="X34" s="10"/>
+      <c r="Y34" s="10"/>
+      <c r="Z34" s="10"/>
+      <c r="AA34" s="10"/>
+    </row>
+    <row r="35" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>46366</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q35" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S35" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="T35" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U35" s="9"/>
+      <c r="V35" s="10"/>
+      <c r="W35" s="10"/>
+      <c r="X35" s="10"/>
+      <c r="Y35" s="10"/>
+      <c r="Z35" s="10"/>
+      <c r="AA35" s="10"/>
+    </row>
+    <row r="36" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>46368</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="T36" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U36" s="9"/>
+      <c r="V36" s="10"/>
+      <c r="W36" s="10"/>
+      <c r="X36" s="10"/>
+      <c r="Y36" s="10"/>
+      <c r="Z36" s="10"/>
+      <c r="AA36" s="10"/>
+    </row>
+    <row r="37" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>46369</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="M37" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="N37" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q37" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="T37" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="U37" s="9"/>
+      <c r="V37" s="10"/>
+      <c r="W37" s="10"/>
+      <c r="X37" s="10"/>
+      <c r="Y37" s="10"/>
+      <c r="Z37" s="10"/>
+      <c r="AA37" s="10"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA21"/>
+  <autoFilter ref="A1:AA37"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="T2:T21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="T2:T37" type="list">
       <formula1>"Planned,Filmed,Edited,Scheduled,Posted,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3148,84 +4598,84 @@
         <v>18</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>176</v>
+        <v>247</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>177</v>
+        <v>248</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>178</v>
+        <v>249</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>179</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>180</v>
+        <v>251</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>181</v>
+        <v>252</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>182</v>
+        <v>253</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>181</v>
+        <v>252</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>183</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>184</v>
+        <v>255</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>185</v>
+        <v>256</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>186</v>
+        <v>257</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>187</v>
+        <v>258</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>188</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>189</v>
+        <v>260</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>190</v>
+        <v>261</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>191</v>
+        <v>262</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>192</v>
+        <v>263</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>193</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>194</v>
+        <v>265</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>195</v>
+        <v>266</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>196</v>
+        <v>267</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>197</v>
+        <v>268</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>198</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3253,82 +4703,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>199</v>
+        <v>270</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>200</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>201</v>
+        <v>272</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>202</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>203</v>
+        <v>274</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>204</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>205</v>
+        <v>276</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>206</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>207</v>
+        <v>278</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>208</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>209</v>
+        <v>280</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>210</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>211</v>
+        <v>282</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>212</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>213</v>
+        <v>284</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>214</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>215</v>
+        <v>286</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>216</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>217</v>
+        <v>288</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>218</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -3347,7 +4797,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -3359,19 +4809,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>219</v>
+        <v>290</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>220</v>
+        <v>291</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>222</v>
+        <v>293</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>223</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3382,64 +4832,149 @@
         <v>46313</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>224</v>
+        <v>295</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>225</v>
+        <v>296</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>226</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>118</v>
+        <v>77</v>
       </c>
       <c r="B3" s="7" t="n">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>227</v>
+        <v>298</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>228</v>
+        <v>299</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>229</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="B4" s="7" t="n">
-        <v>46332</v>
+        <v>46319</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>230</v>
+        <v>301</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>231</v>
+        <v>302</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>226</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>77</v>
+        <v>163</v>
       </c>
       <c r="B5" s="7" t="n">
-        <v>46314</v>
+        <v>46332</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>232</v>
+        <v>303</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>233</v>
+        <v>304</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>229</v>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>46340</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>46347</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>46354</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>46361</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>46341</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -3458,7 +4993,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3477,13 +5012,13 @@
         <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>234</v>
+        <v>315</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>235</v>
+        <v>316</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>236</v>
+        <v>317</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>37</v>
@@ -3504,10 +5039,10 @@
         <v>42</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>237</v>
+        <v>318</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>238</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3518,35 +5053,35 @@
         <v>46307</v>
       </c>
       <c r="C2" s="14" t="n">
-        <f aca="false">COUNTIF(Calendar!$A$2:$A$21,A2)</f>
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A2)</f>
         <v>4</v>
       </c>
       <c r="D2" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A2,Calendar!$T$2:$T$21,"Posted")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A2,Calendar!$T$2:$T$37,"Posted")</f>
+        <v>3</v>
       </c>
       <c r="E2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$V$2:$V$37)</f>
         <v>0</v>
       </c>
       <c r="F2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$W$2:$W$37)</f>
         <v>0</v>
       </c>
       <c r="G2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$X$2:$X$37)</f>
         <v>0</v>
       </c>
       <c r="H2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$Y$2:$Y$37)</f>
         <v>0</v>
       </c>
       <c r="I2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$Z$2:$Z$37)</f>
         <v>0</v>
       </c>
       <c r="J2" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A2,Calendar!$AA$2:$AA$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A2,Calendar!$AA$2:$AA$37)</f>
         <v>0</v>
       </c>
       <c r="K2" s="17" t="n">
@@ -3563,35 +5098,35 @@
         <v>46314</v>
       </c>
       <c r="C3" s="14" t="n">
-        <f aca="false">COUNTIF(Calendar!$A$2:$A$21,A3)</f>
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A3)</f>
         <v>4</v>
       </c>
       <c r="D3" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A3,Calendar!$T$2:$T$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A3,Calendar!$T$2:$T$37,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$V$2:$V$37)</f>
         <v>0</v>
       </c>
       <c r="F3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$W$2:$W$37)</f>
         <v>0</v>
       </c>
       <c r="G3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$X$2:$X$37)</f>
         <v>0</v>
       </c>
       <c r="H3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$Y$2:$Y$37)</f>
         <v>0</v>
       </c>
       <c r="I3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$Z$2:$Z$37)</f>
         <v>0</v>
       </c>
       <c r="J3" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A3,Calendar!$AA$2:$AA$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A3,Calendar!$AA$2:$AA$37)</f>
         <v>0</v>
       </c>
       <c r="K3" s="17" t="n">
@@ -3608,35 +5143,35 @@
         <v>46321</v>
       </c>
       <c r="C4" s="14" t="n">
-        <f aca="false">COUNTIF(Calendar!$A$2:$A$21,A4)</f>
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A4)</f>
         <v>4</v>
       </c>
       <c r="D4" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A4,Calendar!$T$2:$T$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A4,Calendar!$T$2:$T$37,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$V$2:$V$37)</f>
         <v>0</v>
       </c>
       <c r="F4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$W$2:$W$37)</f>
         <v>0</v>
       </c>
       <c r="G4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$X$2:$X$37)</f>
         <v>0</v>
       </c>
       <c r="H4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$Y$2:$Y$37)</f>
         <v>0</v>
       </c>
       <c r="I4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$Z$2:$Z$37)</f>
         <v>0</v>
       </c>
       <c r="J4" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A4,Calendar!$AA$2:$AA$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A4,Calendar!$AA$2:$AA$37)</f>
         <v>0</v>
       </c>
       <c r="K4" s="17" t="n">
@@ -3653,35 +5188,35 @@
         <v>46328</v>
       </c>
       <c r="C5" s="14" t="n">
-        <f aca="false">COUNTIF(Calendar!$A$2:$A$21,A5)</f>
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A5)</f>
         <v>4</v>
       </c>
       <c r="D5" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A5,Calendar!$T$2:$T$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A5,Calendar!$T$2:$T$37,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$V$2:$V$37)</f>
         <v>0</v>
       </c>
       <c r="F5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$W$2:$W$37)</f>
         <v>0</v>
       </c>
       <c r="G5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$X$2:$X$37)</f>
         <v>0</v>
       </c>
       <c r="H5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$Y$2:$Y$37)</f>
         <v>0</v>
       </c>
       <c r="I5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$Z$2:$Z$37)</f>
         <v>0</v>
       </c>
       <c r="J5" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A5,Calendar!$AA$2:$AA$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A5,Calendar!$AA$2:$AA$37)</f>
         <v>0</v>
       </c>
       <c r="K5" s="17" t="n">
@@ -3698,35 +5233,35 @@
         <v>46335</v>
       </c>
       <c r="C6" s="14" t="n">
-        <f aca="false">COUNTIF(Calendar!$A$2:$A$21,A6)</f>
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A6)</f>
         <v>4</v>
       </c>
       <c r="D6" s="14" t="n">
-        <f aca="false">COUNTIFS(Calendar!$A$2:$A$21,A6,Calendar!$T$2:$T$21,"Posted")</f>
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A6,Calendar!$T$2:$T$37,"Posted")</f>
         <v>0</v>
       </c>
       <c r="E6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$V$2:$V$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$V$2:$V$37)</f>
         <v>0</v>
       </c>
       <c r="F6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$W$2:$W$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$W$2:$W$37)</f>
         <v>0</v>
       </c>
       <c r="G6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$X$2:$X$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$X$2:$X$37)</f>
         <v>0</v>
       </c>
       <c r="H6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Y$2:$Y$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$Y$2:$Y$37)</f>
         <v>0</v>
       </c>
       <c r="I6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$Z$2:$Z$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$Z$2:$Z$37)</f>
         <v>0</v>
       </c>
       <c r="J6" s="16" t="n">
-        <f aca="false">SUMIF(Calendar!$A$2:$A$21,A6,Calendar!$AA$2:$AA$21)</f>
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A6,Calendar!$AA$2:$AA$37)</f>
         <v>0</v>
       </c>
       <c r="K6" s="17" t="n">
@@ -3736,49 +5271,229 @@
       <c r="L6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="C7" s="19" t="n">
-        <f aca="false">SUM(C2:C6)</f>
-        <v>20</v>
-      </c>
-      <c r="D7" s="19" t="n">
-        <f aca="false">SUM(D2:D6)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <f aca="false">SUM(E2:E6)</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <f aca="false">SUM(F2:F6)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <f aca="false">SUM(G2:G6)</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <f aca="false">SUM(H2:H6)</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <f aca="false">SUM(I2:I6)</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="19" t="n">
-        <f aca="false">SUM(J2:J6)</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="20" t="n">
+      <c r="A7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>46342</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A7)</f>
+        <v>4</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A7,Calendar!$T$2:$T$37,"Posted")</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$V$2:$V$37)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$W$2:$W$37)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$X$2:$X$37)</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$Y$2:$Y$37)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$Z$2:$Z$37)</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A7,Calendar!$AA$2:$AA$37)</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="17" t="n">
         <f aca="false">IFERROR(G7/E7*1000,0)</f>
         <v>0</v>
       </c>
+      <c r="L7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>46349</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A8)</f>
+        <v>4</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A8,Calendar!$T$2:$T$37,"Posted")</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$V$2:$V$37)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$W$2:$W$37)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$X$2:$X$37)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$Y$2:$Y$37)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$Z$2:$Z$37)</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A8,Calendar!$AA$2:$AA$37)</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <f aca="false">IFERROR(G8/E8*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>240</v>
+      <c r="A9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>46356</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A9)</f>
+        <v>4</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A9,Calendar!$T$2:$T$37,"Posted")</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$V$2:$V$37)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$W$2:$W$37)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$X$2:$X$37)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$Y$2:$Y$37)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$Z$2:$Z$37)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A9,Calendar!$AA$2:$AA$37)</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <f aca="false">IFERROR(G9/E9*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>46363</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <f aca="false">COUNTIF(Calendar!$A$2:$A$37,A10)</f>
+        <v>4</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <f aca="false">COUNTIFS(Calendar!$A$2:$A$37,A10,Calendar!$T$2:$T$37,"Posted")</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$V$2:$V$37)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$W$2:$W$37)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$X$2:$X$37)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$Y$2:$Y$37)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$Z$2:$Z$37)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <f aca="false">SUMIF(Calendar!$A$2:$A$37,A10,Calendar!$AA$2:$AA$37)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <f aca="false">IFERROR(G10/E10*1000,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <f aca="false">SUM(C2:C10)</f>
+        <v>36</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <f aca="false">SUM(D2:D10)</f>
+        <v>3</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <f aca="false">SUM(E2:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <f aca="false">SUM(F2:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <f aca="false">SUM(G2:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <f aca="false">SUM(H2:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <f aca="false">SUM(I2:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <f aca="false">SUM(J2:J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="20" t="n">
+        <f aca="false">IFERROR(G11/E11*1000,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -3807,94 +5522,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>241</v>
+        <v>322</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>242</v>
+        <v>323</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>179</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22"/>
       <c r="B2" s="6" t="s">
-        <v>243</v>
+        <v>324</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>244</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22"/>
       <c r="B3" s="6" t="s">
-        <v>245</v>
+        <v>326</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>246</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22"/>
       <c r="B4" s="6" t="s">
-        <v>247</v>
+        <v>328</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>248</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22"/>
       <c r="B5" s="6" t="s">
-        <v>249</v>
+        <v>330</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>250</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22"/>
       <c r="B6" s="6" t="s">
-        <v>251</v>
+        <v>332</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
-        <v>253</v>
+        <v>334</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>254</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
-        <v>255</v>
+        <v>336</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>256</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
-        <v>257</v>
+        <v>338</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>258</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22"/>
       <c r="B10" s="6" t="s">
-        <v>259</v>
+        <v>340</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>260</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>